<commit_message>
Fixed Parent meter serial
</commit_message>
<xml_diff>
--- a/EVG_Lake_Michelle_Meter_Hierarchy_2026-07-03.xlsx
+++ b/EVG_Lake_Michelle_Meter_Hierarchy_2026-07-03.xlsx
@@ -5,16 +5,19 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://voltano-my.sharepoint.com/personal/ruan_vh_voltano_com/Documents/Desktop/Voltano/Clients/Evergreen/Lake Michelle Noordhoek/Site Commissioning/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://voltano-my.sharepoint.com/personal/ruan_vh_voltano_com/Documents/Desktop/Voltano/Clients/Evergreen/Lake Michelle Noordhoek/Site Management/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="272" documentId="8_{E5281369-C957-4F01-BD7F-34BF193967CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{167C0BA4-2F16-496B-A649-E1D2B7ED428E}"/>
+  <xr:revisionPtr revIDLastSave="285" documentId="8_{E5281369-C957-4F01-BD7F-34BF193967CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{71B29E43-64FA-4062-BEE6-EEEEEF8E37FC}"/>
   <bookViews>
     <workbookView xWindow="71880" yWindow="-1530" windowWidth="29040" windowHeight="15720" xr2:uid="{AE166FFD-83CC-4E71-A293-C6082B1A6C83}"/>
   </bookViews>
   <sheets>
     <sheet name="Elec" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Elec!$A$1:$L$87</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -526,7 +529,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -572,24 +575,11 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="9">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="8">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1066,7 +1056,7 @@
       <c r="K1" s="10" t="s">
         <v>124</v>
       </c>
-      <c r="L1" s="14" t="s">
+      <c r="L1" s="10" t="s">
         <v>128</v>
       </c>
     </row>
@@ -1510,7 +1500,7 @@
         <v>91732797</v>
       </c>
       <c r="C14" s="2">
-        <v>98820079</v>
+        <v>98820081</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>116</v>
@@ -1546,7 +1536,7 @@
         <v>91732835</v>
       </c>
       <c r="C15" s="2">
-        <v>98820079</v>
+        <v>98820081</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>116</v>
@@ -1582,7 +1572,7 @@
         <v>91546283</v>
       </c>
       <c r="C16" s="2">
-        <v>98820079</v>
+        <v>98820081</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>116</v>
@@ -1618,7 +1608,7 @@
         <v>91732806</v>
       </c>
       <c r="C17" s="2">
-        <v>98820079</v>
+        <v>98820081</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>116</v>
@@ -1654,7 +1644,7 @@
         <v>91732775</v>
       </c>
       <c r="C18" s="2">
-        <v>98820079</v>
+        <v>98820081</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>116</v>
@@ -1690,7 +1680,7 @@
         <v>91732809</v>
       </c>
       <c r="C19" s="2">
-        <v>98820081</v>
+        <v>98820079</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>116</v>
@@ -1726,7 +1716,7 @@
         <v>91732788</v>
       </c>
       <c r="C20" s="2">
-        <v>98820081</v>
+        <v>98820079</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>116</v>
@@ -1762,7 +1752,7 @@
         <v>91546333</v>
       </c>
       <c r="C21" s="2">
-        <v>98820081</v>
+        <v>98820079</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>116</v>
@@ -1798,7 +1788,7 @@
         <v>91732814</v>
       </c>
       <c r="C22" s="2">
-        <v>98820081</v>
+        <v>98820079</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>116</v>
@@ -1834,7 +1824,7 @@
         <v>91732831</v>
       </c>
       <c r="C23" s="2">
-        <v>98820079</v>
+        <v>98820081</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>116</v>
@@ -1870,7 +1860,7 @@
         <v>91732781</v>
       </c>
       <c r="C24" s="2">
-        <v>98820079</v>
+        <v>98820081</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>116</v>
@@ -1906,7 +1896,7 @@
         <v>91732815</v>
       </c>
       <c r="C25" s="2">
-        <v>98820079</v>
+        <v>98820081</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>116</v>
@@ -1942,7 +1932,7 @@
         <v>91732780</v>
       </c>
       <c r="C26" s="2">
-        <v>98820079</v>
+        <v>98820081</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>116</v>
@@ -1978,7 +1968,7 @@
         <v>91732841</v>
       </c>
       <c r="C27" s="2">
-        <v>98820079</v>
+        <v>98820081</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>116</v>
@@ -2014,7 +2004,7 @@
         <v>91732795</v>
       </c>
       <c r="C28" s="2">
-        <v>98820081</v>
+        <v>98820079</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>116</v>
@@ -2050,7 +2040,7 @@
         <v>91546331</v>
       </c>
       <c r="C29" s="2">
-        <v>98820081</v>
+        <v>98820079</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>116</v>
@@ -2086,7 +2076,7 @@
         <v>91732836</v>
       </c>
       <c r="C30" s="2">
-        <v>98820081</v>
+        <v>98820079</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>116</v>
@@ -2122,7 +2112,7 @@
         <v>91732802</v>
       </c>
       <c r="C31" s="2">
-        <v>98820081</v>
+        <v>98820079</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>116</v>
@@ -2194,7 +2184,7 @@
         <v>91546282</v>
       </c>
       <c r="C33" s="2">
-        <v>98820081</v>
+        <v>98820079</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>116</v>
@@ -2232,7 +2222,7 @@
         <v>91732791</v>
       </c>
       <c r="C34" s="2">
-        <v>98820081</v>
+        <v>98820079</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>116</v>
@@ -2270,7 +2260,7 @@
         <v>91732818</v>
       </c>
       <c r="C35" s="2">
-        <v>98820081</v>
+        <v>98820079</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>116</v>
@@ -2308,7 +2298,7 @@
         <v>91732782</v>
       </c>
       <c r="C36" s="2">
-        <v>98820081</v>
+        <v>98820079</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>116</v>
@@ -2346,7 +2336,7 @@
         <v>91546307</v>
       </c>
       <c r="C37" s="2">
-        <v>98820081</v>
+        <v>98820079</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>116</v>
@@ -2384,7 +2374,7 @@
         <v>91732842</v>
       </c>
       <c r="C38" s="2">
-        <v>98820079</v>
+        <v>98820081</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>116</v>
@@ -2420,7 +2410,7 @@
         <v>91732793</v>
       </c>
       <c r="C39" s="2">
-        <v>98820079</v>
+        <v>98820081</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>116</v>
@@ -2456,7 +2446,7 @@
         <v>91732840</v>
       </c>
       <c r="C40" s="2">
-        <v>98820079</v>
+        <v>98820081</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>116</v>
@@ -2492,7 +2482,7 @@
         <v>91732817</v>
       </c>
       <c r="C41" s="2">
-        <v>98820079</v>
+        <v>98820081</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>116</v>
@@ -2528,7 +2518,7 @@
         <v>91732792</v>
       </c>
       <c r="C42" s="2">
-        <v>98820079</v>
+        <v>98820081</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>116</v>
@@ -2564,7 +2554,7 @@
         <v>91732796</v>
       </c>
       <c r="C43" s="2">
-        <v>98820079</v>
+        <v>98820081</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>116</v>
@@ -2600,7 +2590,7 @@
         <v>91546227</v>
       </c>
       <c r="C44" s="2">
-        <v>98820081</v>
+        <v>98820079</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>116</v>
@@ -2638,7 +2628,7 @@
         <v>91732786</v>
       </c>
       <c r="C45" s="2">
-        <v>98820081</v>
+        <v>98820079</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>116</v>
@@ -2676,7 +2666,7 @@
         <v>91732808</v>
       </c>
       <c r="C46" s="2">
-        <v>98820081</v>
+        <v>98820079</v>
       </c>
       <c r="D46" s="2" t="s">
         <v>116</v>
@@ -2714,7 +2704,7 @@
         <v>91546277</v>
       </c>
       <c r="C47" s="2">
-        <v>98820081</v>
+        <v>98820079</v>
       </c>
       <c r="D47" s="2" t="s">
         <v>116</v>
@@ -2752,7 +2742,7 @@
         <v>91732798</v>
       </c>
       <c r="C48" s="2">
-        <v>98820081</v>
+        <v>98820079</v>
       </c>
       <c r="D48" s="2" t="s">
         <v>116</v>
@@ -2790,7 +2780,7 @@
         <v>91732794</v>
       </c>
       <c r="C49" s="2">
-        <v>98820079</v>
+        <v>98820081</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>116</v>
@@ -2826,7 +2816,7 @@
         <v>91732774</v>
       </c>
       <c r="C50" s="2">
-        <v>98820079</v>
+        <v>98820081</v>
       </c>
       <c r="D50" s="2" t="s">
         <v>116</v>
@@ -2862,7 +2852,7 @@
         <v>91732776</v>
       </c>
       <c r="C51" s="2">
-        <v>98820079</v>
+        <v>98820081</v>
       </c>
       <c r="D51" s="2" t="s">
         <v>116</v>
@@ -2898,7 +2888,7 @@
         <v>91732801</v>
       </c>
       <c r="C52" s="2">
-        <v>98820079</v>
+        <v>98820081</v>
       </c>
       <c r="D52" s="2" t="s">
         <v>116</v>
@@ -2934,7 +2924,7 @@
         <v>91732784</v>
       </c>
       <c r="C53" s="2">
-        <v>98820079</v>
+        <v>98820081</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>116</v>
@@ -2970,7 +2960,7 @@
         <v>91732790</v>
       </c>
       <c r="C54" s="2">
-        <v>98820079</v>
+        <v>98820081</v>
       </c>
       <c r="D54" s="2" t="s">
         <v>116</v>
@@ -3006,7 +2996,7 @@
         <v>91546303</v>
       </c>
       <c r="C55" s="2">
-        <v>98820081</v>
+        <v>98820079</v>
       </c>
       <c r="D55" s="2" t="s">
         <v>116</v>
@@ -3044,7 +3034,7 @@
         <v>91546278</v>
       </c>
       <c r="C56" s="2">
-        <v>98820081</v>
+        <v>98820079</v>
       </c>
       <c r="D56" s="2" t="s">
         <v>116</v>
@@ -3082,7 +3072,7 @@
         <v>91542774</v>
       </c>
       <c r="C57" s="2">
-        <v>98820081</v>
+        <v>98820079</v>
       </c>
       <c r="D57" s="2" t="s">
         <v>116</v>
@@ -3120,7 +3110,7 @@
         <v>91732833</v>
       </c>
       <c r="C58" s="2">
-        <v>98820081</v>
+        <v>98820079</v>
       </c>
       <c r="D58" s="2" t="s">
         <v>116</v>
@@ -3158,7 +3148,7 @@
         <v>91732778</v>
       </c>
       <c r="C59" s="2">
-        <v>98820081</v>
+        <v>98820079</v>
       </c>
       <c r="D59" s="2" t="s">
         <v>116</v>
@@ -3196,7 +3186,7 @@
         <v>91546300</v>
       </c>
       <c r="C60" s="2">
-        <v>98820079</v>
+        <v>98820081</v>
       </c>
       <c r="D60" s="2" t="s">
         <v>116</v>
@@ -3232,7 +3222,7 @@
         <v>91732839</v>
       </c>
       <c r="C61" s="2">
-        <v>98820079</v>
+        <v>98820081</v>
       </c>
       <c r="D61" s="2" t="s">
         <v>116</v>
@@ -3268,7 +3258,7 @@
         <v>91546308</v>
       </c>
       <c r="C62" s="2">
-        <v>98820079</v>
+        <v>98820081</v>
       </c>
       <c r="D62" s="2" t="s">
         <v>116</v>
@@ -3304,7 +3294,7 @@
         <v>91732813</v>
       </c>
       <c r="C63" s="2">
-        <v>98820079</v>
+        <v>98820081</v>
       </c>
       <c r="D63" s="2" t="s">
         <v>116</v>
@@ -3556,7 +3546,7 @@
         <v>91732773</v>
       </c>
       <c r="C70" s="2">
-        <v>98820079</v>
+        <v>98820081</v>
       </c>
       <c r="D70" s="2" t="s">
         <v>116</v>
@@ -3592,7 +3582,7 @@
         <v>91732810</v>
       </c>
       <c r="C71" s="2">
-        <v>98820079</v>
+        <v>98820081</v>
       </c>
       <c r="D71" s="2" t="s">
         <v>116</v>
@@ -3628,7 +3618,7 @@
         <v>91732787</v>
       </c>
       <c r="C72" s="2">
-        <v>98820079</v>
+        <v>98820081</v>
       </c>
       <c r="D72" s="2" t="s">
         <v>116</v>
@@ -3664,7 +3654,7 @@
         <v>91732771</v>
       </c>
       <c r="C73" s="2">
-        <v>98820079</v>
+        <v>98820081</v>
       </c>
       <c r="D73" s="2" t="s">
         <v>116</v>
@@ -3738,7 +3728,7 @@
         <v>91732783</v>
       </c>
       <c r="C75" s="2">
-        <v>98820081</v>
+        <v>98820079</v>
       </c>
       <c r="D75" s="2" t="s">
         <v>116</v>
@@ -3776,7 +3766,7 @@
         <v>91732779</v>
       </c>
       <c r="C76" s="2">
-        <v>98820081</v>
+        <v>98820079</v>
       </c>
       <c r="D76" s="2" t="s">
         <v>116</v>
@@ -3814,7 +3804,7 @@
         <v>91732789</v>
       </c>
       <c r="C77" s="2">
-        <v>98820081</v>
+        <v>98820079</v>
       </c>
       <c r="D77" s="2" t="s">
         <v>116</v>
@@ -3852,7 +3842,7 @@
         <v>91546253</v>
       </c>
       <c r="C78" s="2">
-        <v>98820081</v>
+        <v>98820079</v>
       </c>
       <c r="D78" s="2" t="s">
         <v>116</v>
@@ -3926,7 +3916,7 @@
         <v>91546325</v>
       </c>
       <c r="C80" s="2">
-        <v>98820081</v>
+        <v>98820079</v>
       </c>
       <c r="D80" s="2" t="s">
         <v>116</v>
@@ -3962,7 +3952,7 @@
         <v>91732805</v>
       </c>
       <c r="C81" s="2">
-        <v>98820081</v>
+        <v>98820079</v>
       </c>
       <c r="D81" s="2" t="s">
         <v>116</v>
@@ -3998,7 +3988,7 @@
         <v>91732800</v>
       </c>
       <c r="C82" s="2">
-        <v>98820081</v>
+        <v>98820079</v>
       </c>
       <c r="D82" s="2" t="s">
         <v>116</v>
@@ -4211,10 +4201,28 @@
     <sortCondition ref="H2:H87"/>
   </sortState>
   <phoneticPr fontId="3" type="noConversion"/>
+  <conditionalFormatting sqref="A2:A87">
+    <cfRule type="duplicateValues" dxfId="7" priority="7"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B2:B87">
+    <cfRule type="duplicateValues" dxfId="6" priority="8"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C79:C84">
+    <cfRule type="duplicateValues" dxfId="5" priority="6"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C74:C78">
+    <cfRule type="duplicateValues" dxfId="4" priority="5"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C64:C69">
+    <cfRule type="duplicateValues" dxfId="3" priority="4"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C55:C59">
+    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C44:C48 C33:C37 C28:C31 C19:C22 C2:C13">
     <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:A87">
+  <conditionalFormatting sqref="C70:C73 C60:C63 C49:C54 C38:C43 C32 C23:C27 C14:C18">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
New AMR installed, updating the list
</commit_message>
<xml_diff>
--- a/EVG_Lake_Michelle_Meter_Hierarchy_2026-07-03.xlsx
+++ b/EVG_Lake_Michelle_Meter_Hierarchy_2026-07-03.xlsx
@@ -8,13 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://voltano-my.sharepoint.com/personal/ruan_vh_voltano_com/Documents/Desktop/Voltano/Clients/Evergreen/Lake Michelle Noordhoek/Site Management/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="337" documentId="8_{E5281369-C957-4F01-BD7F-34BF193967CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F04A4E19-B74D-40D7-87E6-315078472909}"/>
+  <xr:revisionPtr revIDLastSave="338" documentId="8_{E5281369-C957-4F01-BD7F-34BF193967CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E585B5A4-73B9-4B82-A03A-89908CC90E51}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{AE166FFD-83CC-4E71-A293-C6082B1A6C83}"/>
+    <workbookView xWindow="8010" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{AE166FFD-83CC-4E71-A293-C6082B1A6C83}"/>
   </bookViews>
   <sheets>
     <sheet name="Elec" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Elec!$A$1:$L$87</definedName>
@@ -442,10 +441,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="44" formatCode="_-&quot;R&quot;* #,##0.00_-;\-&quot;R&quot;* #,##0.00_-;_-&quot;R&quot;* &quot;-&quot;??_-;_-@_-"/>
-  </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -470,13 +466,6 @@
     </font>
     <font>
       <sz val="8"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -543,11 +532,10 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -593,10 +581,8 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Currency" xfId="1" builtinId="4"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="2">
@@ -4190,20 +4176,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EA7687B-358E-412C-9E41-3D320E9423EE}">
-  <dimension ref="D16"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <cols>
-    <col min="4" max="4" width="13.6640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="16" spans="4:4" x14ac:dyDescent="0.45">
-      <c r="D16" s="14"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
New tab added for Updated Stand
</commit_message>
<xml_diff>
--- a/EVG_Lake_Michelle_Meter_Hierarchy_2026-07-03.xlsx
+++ b/EVG_Lake_Michelle_Meter_Hierarchy_2026-07-03.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://voltano-my.sharepoint.com/personal/ruan_vh_voltano_com/Documents/Desktop/Voltano/Clients/Evergreen/Lake Michelle Noordhoek/Site Management/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="478" documentId="8_{E5281369-C957-4F01-BD7F-34BF193967CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{837DAC2E-D36F-460F-B0BB-E0B3E7679169}"/>
+  <xr:revisionPtr revIDLastSave="508" documentId="8_{E5281369-C957-4F01-BD7F-34BF193967CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BAEAEE14-7A4C-4D9A-9DDE-707AA2F256F6}"/>
   <bookViews>
-    <workbookView xWindow="8010" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{AE166FFD-83CC-4E71-A293-C6082B1A6C83}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{AE166FFD-83CC-4E71-A293-C6082B1A6C83}"/>
   </bookViews>
   <sheets>
     <sheet name="Elec" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="532" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="533" uniqueCount="135">
   <si>
     <t>Stand Number</t>
   </si>
@@ -444,6 +444,9 @@
   </si>
   <si>
     <t>57</t>
+  </si>
+  <si>
+    <t>Stand Updated</t>
   </si>
 </sst>
 </file>
@@ -544,7 +547,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -588,6 +591,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -962,7 +968,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE70038C-F77E-467C-8590-F4D9FE8E81E9}">
-  <dimension ref="A1:L87"/>
+  <dimension ref="A1:M87"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="13" bestFit="1" customWidth="1"/>
@@ -974,10 +980,11 @@
     <col min="9" max="9" width="20.46484375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="24.33203125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12.46484375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.46484375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.3984375" customWidth="1"/>
+    <col min="13" max="13" width="12.3984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1014,8 +1021,11 @@
       <c r="L1" s="10" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M1" s="14" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A2" s="3" t="s">
         <v>108</v>
       </c>
@@ -1052,8 +1062,11 @@
       <c r="L2" s="2">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M2" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
         <v>107</v>
       </c>
@@ -1090,8 +1103,11 @@
       <c r="L3" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M3" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
         <v>106</v>
       </c>
@@ -1128,8 +1144,11 @@
       <c r="L4" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M4" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A5" s="3" t="s">
         <v>109</v>
       </c>
@@ -1166,8 +1185,11 @@
       <c r="L5" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M5" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A6" s="3" t="s">
         <v>110</v>
       </c>
@@ -1204,8 +1226,11 @@
       <c r="L6" s="2">
         <v>5</v>
       </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M6" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A7" s="3" t="s">
         <v>111</v>
       </c>
@@ -1242,8 +1267,11 @@
       <c r="L7" s="2">
         <v>6</v>
       </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M7" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A8" s="3" t="s">
         <v>113</v>
       </c>
@@ -1280,8 +1308,11 @@
       <c r="L8" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M8" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A9" s="3" t="s">
         <v>114</v>
       </c>
@@ -1318,8 +1349,11 @@
       <c r="L9" s="2">
         <v>3</v>
       </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M9" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A10" s="3" t="s">
         <v>112</v>
       </c>
@@ -1356,8 +1390,11 @@
       <c r="L10" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M10" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A11" s="3" t="s">
         <v>115</v>
       </c>
@@ -1394,8 +1431,11 @@
       <c r="L11" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M11" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A12" s="3" t="s">
         <v>116</v>
       </c>
@@ -1432,8 +1472,11 @@
       <c r="L12" s="2">
         <v>5</v>
       </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M12" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A13" s="3" t="s">
         <v>117</v>
       </c>
@@ -1470,8 +1513,11 @@
       <c r="L13" s="2">
         <v>6</v>
       </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M13" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A14" s="3" t="s">
         <v>121</v>
       </c>
@@ -1508,8 +1554,11 @@
       <c r="L14" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M14" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A15" s="3" t="s">
         <v>120</v>
       </c>
@@ -1546,8 +1595,11 @@
       <c r="L15" s="2">
         <v>3</v>
       </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M15" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A16" s="3" t="s">
         <v>119</v>
       </c>
@@ -1584,8 +1636,11 @@
       <c r="L16" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M16" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A17" s="3" t="s">
         <v>118</v>
       </c>
@@ -1622,8 +1677,11 @@
       <c r="L17" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M17" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A18" s="3" t="s">
         <v>122</v>
       </c>
@@ -1660,8 +1718,11 @@
       <c r="L18" s="2">
         <v>5</v>
       </c>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M18" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A19" s="3" t="s">
         <v>79</v>
       </c>
@@ -1696,8 +1757,11 @@
         <v>0</v>
       </c>
       <c r="L19" s="2"/>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M19" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A20" s="3" t="s">
         <v>80</v>
       </c>
@@ -1732,8 +1796,11 @@
         <v>0</v>
       </c>
       <c r="L20" s="2"/>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M20" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A21" s="3" t="s">
         <v>81</v>
       </c>
@@ -1768,8 +1835,11 @@
         <v>0</v>
       </c>
       <c r="L21" s="2"/>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M21" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A22" s="3" t="s">
         <v>82</v>
       </c>
@@ -1804,8 +1874,11 @@
         <v>0</v>
       </c>
       <c r="L22" s="2"/>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M22" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A23" s="3" t="s">
         <v>126</v>
       </c>
@@ -1842,8 +1915,11 @@
       <c r="L23" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M23" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A24" s="3" t="s">
         <v>125</v>
       </c>
@@ -1880,8 +1956,11 @@
       <c r="L24" s="2">
         <v>3</v>
       </c>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M24" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A25" s="3" t="s">
         <v>127</v>
       </c>
@@ -1918,8 +1997,11 @@
       <c r="L25" s="2">
         <v>5</v>
       </c>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M25" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A26" s="3" t="s">
         <v>124</v>
       </c>
@@ -1956,8 +2038,11 @@
       <c r="L26" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M26" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A27" s="3" t="s">
         <v>123</v>
       </c>
@@ -1994,8 +2079,11 @@
       <c r="L27" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M27" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A28" s="3" t="s">
         <v>75</v>
       </c>
@@ -2030,8 +2118,11 @@
         <v>0</v>
       </c>
       <c r="L28" s="2"/>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M28" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A29" s="3" t="s">
         <v>76</v>
       </c>
@@ -2066,8 +2157,11 @@
         <v>0</v>
       </c>
       <c r="L29" s="2"/>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M29" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A30" s="3" t="s">
         <v>77</v>
       </c>
@@ -2102,8 +2196,11 @@
         <v>0</v>
       </c>
       <c r="L30" s="2"/>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M30" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A31" s="3" t="s">
         <v>78</v>
       </c>
@@ -2138,8 +2235,11 @@
         <v>0</v>
       </c>
       <c r="L31" s="2"/>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M31" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A32" s="3" t="s">
         <v>9</v>
       </c>
@@ -2174,8 +2274,11 @@
         <v>0</v>
       </c>
       <c r="L32" s="2"/>
-    </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M32" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A33" s="3" t="s">
         <v>60</v>
       </c>
@@ -2212,8 +2315,11 @@
       <c r="L33" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M33" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A34" s="3" t="s">
         <v>61</v>
       </c>
@@ -2250,8 +2356,11 @@
       <c r="L34" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M34" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A35" s="3" t="s">
         <v>62</v>
       </c>
@@ -2288,8 +2397,11 @@
       <c r="L35" s="2">
         <v>3</v>
       </c>
-    </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M35" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A36" s="3" t="s">
         <v>63</v>
       </c>
@@ -2326,8 +2438,11 @@
       <c r="L36" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M36" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A37" s="3" t="s">
         <v>64</v>
       </c>
@@ -2364,8 +2479,11 @@
       <c r="L37" s="2">
         <v>5</v>
       </c>
-    </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M37" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A38" s="3" t="s">
         <v>130</v>
       </c>
@@ -2402,8 +2520,11 @@
       <c r="L38" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M38" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A39" s="3" t="s">
         <v>129</v>
       </c>
@@ -2440,8 +2561,11 @@
       <c r="L39" s="2">
         <v>3</v>
       </c>
-    </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M39" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A40" s="3" t="s">
         <v>131</v>
       </c>
@@ -2478,8 +2602,11 @@
       <c r="L40" s="2">
         <v>5</v>
       </c>
-    </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M40" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A41" s="3" t="s">
         <v>128</v>
       </c>
@@ -2516,8 +2643,11 @@
       <c r="L41" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M41" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A42" s="3" t="s">
         <v>132</v>
       </c>
@@ -2554,8 +2684,11 @@
       <c r="L42" s="2">
         <v>6</v>
       </c>
-    </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M42" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A43" s="3" t="s">
         <v>133</v>
       </c>
@@ -2592,8 +2725,11 @@
       <c r="L43" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M43" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A44" s="3" t="s">
         <v>65</v>
       </c>
@@ -2630,8 +2766,11 @@
       <c r="L44" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M44" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A45" s="3" t="s">
         <v>66</v>
       </c>
@@ -2668,8 +2807,11 @@
       <c r="L45" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M45" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A46" s="3" t="s">
         <v>67</v>
       </c>
@@ -2706,8 +2848,11 @@
       <c r="L46" s="2">
         <v>3</v>
       </c>
-    </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M46" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A47" s="3" t="s">
         <v>68</v>
       </c>
@@ -2744,8 +2889,11 @@
       <c r="L47" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M47" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A48" s="3" t="s">
         <v>69</v>
       </c>
@@ -2782,8 +2930,11 @@
       <c r="L48" s="2">
         <v>5</v>
       </c>
-    </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M48" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A49" s="3" t="s">
         <v>48</v>
       </c>
@@ -2818,8 +2969,11 @@
         <v>0</v>
       </c>
       <c r="L49" s="2"/>
-    </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M49" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A50" s="3" t="s">
         <v>49</v>
       </c>
@@ -2854,8 +3008,11 @@
         <v>0</v>
       </c>
       <c r="L50" s="2"/>
-    </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M50" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A51" s="3" t="s">
         <v>50</v>
       </c>
@@ -2890,8 +3047,11 @@
         <v>0</v>
       </c>
       <c r="L51" s="2"/>
-    </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M51" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A52" s="3" t="s">
         <v>51</v>
       </c>
@@ -2926,8 +3086,11 @@
         <v>0</v>
       </c>
       <c r="L52" s="2"/>
-    </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M52" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A53" s="3" t="s">
         <v>52</v>
       </c>
@@ -2962,8 +3125,11 @@
         <v>0</v>
       </c>
       <c r="L53" s="2"/>
-    </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M53" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A54" s="3" t="s">
         <v>53</v>
       </c>
@@ -2998,8 +3164,11 @@
         <v>0</v>
       </c>
       <c r="L54" s="2"/>
-    </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M54" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A55" s="3" t="s">
         <v>70</v>
       </c>
@@ -3036,8 +3205,11 @@
       <c r="L55" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M55" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A56" s="3" t="s">
         <v>71</v>
       </c>
@@ -3074,8 +3246,11 @@
       <c r="L56" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M56" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A57" s="3" t="s">
         <v>72</v>
       </c>
@@ -3112,8 +3287,11 @@
       <c r="L57" s="2">
         <v>3</v>
       </c>
-    </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M57" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A58" s="3" t="s">
         <v>73</v>
       </c>
@@ -3150,8 +3328,11 @@
       <c r="L58" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M58" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A59" s="3" t="s">
         <v>74</v>
       </c>
@@ -3188,8 +3369,11 @@
       <c r="L59" s="2">
         <v>5</v>
       </c>
-    </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M59" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A60" s="3" t="s">
         <v>44</v>
       </c>
@@ -3224,8 +3408,11 @@
         <v>0</v>
       </c>
       <c r="L60" s="2"/>
-    </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M60" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A61" s="3" t="s">
         <v>45</v>
       </c>
@@ -3260,8 +3447,11 @@
         <v>0</v>
       </c>
       <c r="L61" s="2"/>
-    </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M61" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A62" s="3" t="s">
         <v>46</v>
       </c>
@@ -3296,8 +3486,11 @@
         <v>0</v>
       </c>
       <c r="L62" s="2"/>
-    </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M62" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A63" s="3" t="s">
         <v>47</v>
       </c>
@@ -3332,8 +3525,11 @@
         <v>0</v>
       </c>
       <c r="L63" s="2"/>
-    </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M63" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A64" s="3" t="s">
         <v>100</v>
       </c>
@@ -3370,8 +3566,11 @@
       <c r="L64" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M64" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A65" s="3" t="s">
         <v>101</v>
       </c>
@@ -3408,8 +3607,11 @@
       <c r="L65" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M65" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A66" s="3" t="s">
         <v>102</v>
       </c>
@@ -3446,8 +3648,11 @@
       <c r="L66" s="2">
         <v>3</v>
       </c>
-    </row>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M66" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A67" s="3" t="s">
         <v>99</v>
       </c>
@@ -3484,8 +3689,11 @@
       <c r="L67" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M67" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A68" s="3" t="s">
         <v>98</v>
       </c>
@@ -3522,8 +3730,11 @@
       <c r="L68" s="2">
         <v>5</v>
       </c>
-    </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M68" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A69" s="3" t="s">
         <v>97</v>
       </c>
@@ -3560,8 +3771,11 @@
       <c r="L69" s="2">
         <v>6</v>
       </c>
-    </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M69" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A70" s="3" t="s">
         <v>40</v>
       </c>
@@ -3596,8 +3810,11 @@
         <v>0</v>
       </c>
       <c r="L70" s="2"/>
-    </row>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M70" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A71" s="3" t="s">
         <v>41</v>
       </c>
@@ -3632,8 +3849,11 @@
         <v>0</v>
       </c>
       <c r="L71" s="2"/>
-    </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M71" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A72" s="3" t="s">
         <v>42</v>
       </c>
@@ -3668,8 +3888,11 @@
         <v>0</v>
       </c>
       <c r="L72" s="2"/>
-    </row>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M72" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A73" s="3" t="s">
         <v>43</v>
       </c>
@@ -3704,8 +3927,11 @@
         <v>0</v>
       </c>
       <c r="L73" s="2"/>
-    </row>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M73" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A74" s="3" t="s">
         <v>54</v>
       </c>
@@ -3742,8 +3968,11 @@
       <c r="L74" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M74" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A75" s="3" t="s">
         <v>58</v>
       </c>
@@ -3780,8 +4009,11 @@
       <c r="L75" s="2">
         <v>5</v>
       </c>
-    </row>
-    <row r="76" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M75" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A76" s="3" t="s">
         <v>57</v>
       </c>
@@ -3818,8 +4050,11 @@
       <c r="L76" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="77" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M76" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A77" s="3" t="s">
         <v>56</v>
       </c>
@@ -3856,8 +4091,11 @@
       <c r="L77" s="2">
         <v>3</v>
       </c>
-    </row>
-    <row r="78" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M77" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A78" s="3" t="s">
         <v>55</v>
       </c>
@@ -3894,8 +4132,11 @@
       <c r="L78" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="79" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M78" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A79" s="3" t="s">
         <v>59</v>
       </c>
@@ -3932,8 +4173,11 @@
       <c r="L79" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="80" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M79" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A80" s="3" t="s">
         <v>103</v>
       </c>
@@ -3970,8 +4214,11 @@
       <c r="L80" s="2">
         <v>3</v>
       </c>
-    </row>
-    <row r="81" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M80" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A81" s="3" t="s">
         <v>104</v>
       </c>
@@ -4008,8 +4255,11 @@
       <c r="L81" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="82" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M81" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A82" s="3" t="s">
         <v>105</v>
       </c>
@@ -4046,8 +4296,11 @@
       <c r="L82" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="83" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M82" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A83" s="3" t="s">
         <v>14</v>
       </c>
@@ -4082,8 +4335,11 @@
         <v>0</v>
       </c>
       <c r="L83" s="2"/>
-    </row>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M83" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A84" s="3" t="s">
         <v>11</v>
       </c>
@@ -4118,8 +4374,11 @@
         <v>0</v>
       </c>
       <c r="L84" s="2"/>
-    </row>
-    <row r="85" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M84" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A85" s="3" t="s">
         <v>37</v>
       </c>
@@ -4154,8 +4413,11 @@
         <v>1</v>
       </c>
       <c r="L85" s="2"/>
-    </row>
-    <row r="86" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M85" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A86" s="3" t="s">
         <v>38</v>
       </c>
@@ -4190,8 +4452,11 @@
         <v>1</v>
       </c>
       <c r="L86" s="2"/>
-    </row>
-    <row r="87" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M86" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="87" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A87" s="3" t="s">
         <v>3</v>
       </c>
@@ -4226,6 +4491,9 @@
         <v>0</v>
       </c>
       <c r="L87" s="2"/>
+      <c r="M87" s="11" t="b">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L87">

</xml_diff>

<commit_message>
New AMR installed and stands relabelled
</commit_message>
<xml_diff>
--- a/EVG_Lake_Michelle_Meter_Hierarchy_2026-07-03.xlsx
+++ b/EVG_Lake_Michelle_Meter_Hierarchy_2026-07-03.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://voltano-my.sharepoint.com/personal/ruan_vh_voltano_com/Documents/Desktop/Voltano/Clients/Evergreen/Lake Michelle Noordhoek/Site Management/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="508" documentId="8_{E5281369-C957-4F01-BD7F-34BF193967CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BAEAEE14-7A4C-4D9A-9DDE-707AA2F256F6}"/>
+  <xr:revisionPtr revIDLastSave="570" documentId="8_{E5281369-C957-4F01-BD7F-34BF193967CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F5D8F626-F6F8-4F6C-8C6D-46B66EFA8383}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{AE166FFD-83CC-4E71-A293-C6082B1A6C83}"/>
   </bookViews>
@@ -176,36 +176,6 @@
     <t>004</t>
   </si>
   <si>
-    <t>005</t>
-  </si>
-  <si>
-    <t>006</t>
-  </si>
-  <si>
-    <t>007</t>
-  </si>
-  <si>
-    <t>008</t>
-  </si>
-  <si>
-    <t>009</t>
-  </si>
-  <si>
-    <t>010</t>
-  </si>
-  <si>
-    <t>011</t>
-  </si>
-  <si>
-    <t>012</t>
-  </si>
-  <si>
-    <t>013</t>
-  </si>
-  <si>
-    <t>014</t>
-  </si>
-  <si>
     <t>036</t>
   </si>
   <si>
@@ -447,6 +417,36 @@
   </si>
   <si>
     <t>Stand Updated</t>
+  </si>
+  <si>
+    <t>73</t>
+  </si>
+  <si>
+    <t>72</t>
+  </si>
+  <si>
+    <t>71</t>
+  </si>
+  <si>
+    <t>62</t>
+  </si>
+  <si>
+    <t>61</t>
+  </si>
+  <si>
+    <t>60</t>
+  </si>
+  <si>
+    <t>63</t>
+  </si>
+  <si>
+    <t>64</t>
+  </si>
+  <si>
+    <t>69</t>
+  </si>
+  <si>
+    <t>70</t>
   </si>
 </sst>
 </file>
@@ -547,7 +547,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -591,9 +591,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -992,13 +989,13 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>5</v>
@@ -1007,27 +1004,27 @@
         <v>2</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="K1" s="10" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="L1" s="10" t="s">
-        <v>96</v>
-      </c>
-      <c r="M1" s="14" t="s">
-        <v>134</v>
+        <v>86</v>
+      </c>
+      <c r="M1" s="10" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A2" s="3" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="B2" s="13">
         <v>91732777</v>
@@ -1036,10 +1033,10 @@
         <v>98820079</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>17</v>
@@ -1068,7 +1065,7 @@
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="B3" s="13">
         <v>91732837</v>
@@ -1077,10 +1074,10 @@
         <v>98820079</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>17</v>
@@ -1109,7 +1106,7 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="B4" s="13">
         <v>91733081</v>
@@ -1118,10 +1115,10 @@
         <v>98820079</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>17</v>
@@ -1150,7 +1147,7 @@
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A5" s="3" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="B5" s="13">
         <v>91732799</v>
@@ -1159,10 +1156,10 @@
         <v>98820079</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>17</v>
@@ -1191,7 +1188,7 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A6" s="3" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="B6" s="13">
         <v>91546302</v>
@@ -1200,10 +1197,10 @@
         <v>98820079</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>17</v>
@@ -1232,7 +1229,7 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A7" s="3" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="B7" s="13">
         <v>91732803</v>
@@ -1241,10 +1238,10 @@
         <v>98820079</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>17</v>
@@ -1273,7 +1270,7 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A8" s="3" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="B8" s="13">
         <v>91546328</v>
@@ -1282,10 +1279,10 @@
         <v>98820079</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>17</v>
@@ -1314,7 +1311,7 @@
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A9" s="3" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="B9" s="13">
         <v>91546327</v>
@@ -1323,10 +1320,10 @@
         <v>98820079</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>17</v>
@@ -1355,7 +1352,7 @@
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A10" s="3" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="B10" s="13">
         <v>91546252</v>
@@ -1364,10 +1361,10 @@
         <v>98820079</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>17</v>
@@ -1396,7 +1393,7 @@
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A11" s="3" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="B11" s="13">
         <v>91732812</v>
@@ -1405,10 +1402,10 @@
         <v>98820079</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>17</v>
@@ -1437,7 +1434,7 @@
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A12" s="3" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="B12" s="13">
         <v>91546326</v>
@@ -1446,10 +1443,10 @@
         <v>98820079</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>17</v>
@@ -1478,7 +1475,7 @@
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A13" s="3" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="B13" s="13">
         <v>91732785</v>
@@ -1487,10 +1484,10 @@
         <v>98820079</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>17</v>
@@ -1519,7 +1516,7 @@
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A14" s="3" t="s">
-        <v>121</v>
+        <v>111</v>
       </c>
       <c r="B14" s="13">
         <v>91732797</v>
@@ -1528,10 +1525,10 @@
         <v>98820081</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>17</v>
@@ -1560,7 +1557,7 @@
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A15" s="3" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="B15" s="13">
         <v>91732835</v>
@@ -1569,10 +1566,10 @@
         <v>98820081</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>17</v>
@@ -1601,7 +1598,7 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A16" s="3" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="B16" s="13">
         <v>91546283</v>
@@ -1610,10 +1607,10 @@
         <v>98820081</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>17</v>
@@ -1642,7 +1639,7 @@
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A17" s="3" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="B17" s="13">
         <v>91732806</v>
@@ -1651,10 +1648,10 @@
         <v>98820081</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>17</v>
@@ -1683,7 +1680,7 @@
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A18" s="3" t="s">
-        <v>122</v>
+        <v>112</v>
       </c>
       <c r="B18" s="13">
         <v>91732775</v>
@@ -1692,10 +1689,10 @@
         <v>98820081</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>17</v>
@@ -1724,7 +1721,7 @@
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A19" s="3" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="B19" s="2">
         <v>91732809</v>
@@ -1733,10 +1730,10 @@
         <v>98820079</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>17</v>
@@ -1763,7 +1760,7 @@
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A20" s="3" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="B20" s="2">
         <v>91732788</v>
@@ -1772,10 +1769,10 @@
         <v>98820079</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>17</v>
@@ -1802,7 +1799,7 @@
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A21" s="3" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B21" s="2">
         <v>91546333</v>
@@ -1811,10 +1808,10 @@
         <v>98820079</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>17</v>
@@ -1841,7 +1838,7 @@
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A22" s="3" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="B22" s="2">
         <v>91732814</v>
@@ -1850,10 +1847,10 @@
         <v>98820079</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>17</v>
@@ -1880,7 +1877,7 @@
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A23" s="3" t="s">
-        <v>126</v>
+        <v>116</v>
       </c>
       <c r="B23" s="13">
         <v>91732831</v>
@@ -1889,10 +1886,10 @@
         <v>98820081</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F23" s="2" t="s">
         <v>17</v>
@@ -1921,7 +1918,7 @@
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A24" s="3" t="s">
-        <v>125</v>
+        <v>115</v>
       </c>
       <c r="B24" s="13">
         <v>91732781</v>
@@ -1930,10 +1927,10 @@
         <v>98820081</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>17</v>
@@ -1962,7 +1959,7 @@
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A25" s="3" t="s">
-        <v>127</v>
+        <v>117</v>
       </c>
       <c r="B25" s="13">
         <v>91732815</v>
@@ -1971,10 +1968,10 @@
         <v>98820081</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>17</v>
@@ -2003,7 +2000,7 @@
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A26" s="3" t="s">
-        <v>124</v>
+        <v>114</v>
       </c>
       <c r="B26" s="13">
         <v>91732780</v>
@@ -2012,10 +2009,10 @@
         <v>98820081</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F26" s="2" t="s">
         <v>17</v>
@@ -2044,7 +2041,7 @@
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A27" s="3" t="s">
-        <v>123</v>
+        <v>113</v>
       </c>
       <c r="B27" s="13">
         <v>91732841</v>
@@ -2053,10 +2050,10 @@
         <v>98820081</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F27" s="2" t="s">
         <v>17</v>
@@ -2085,7 +2082,7 @@
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A28" s="3" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="B28" s="4">
         <v>91732795</v>
@@ -2094,10 +2091,10 @@
         <v>98820079</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F28" s="2" t="s">
         <v>17</v>
@@ -2124,7 +2121,7 @@
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A29" s="3" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="B29" s="4">
         <v>91546331</v>
@@ -2133,10 +2130,10 @@
         <v>98820079</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F29" s="2" t="s">
         <v>17</v>
@@ -2163,7 +2160,7 @@
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A30" s="3" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="B30" s="4">
         <v>91732836</v>
@@ -2172,10 +2169,10 @@
         <v>98820079</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F30" s="2" t="s">
         <v>17</v>
@@ -2202,7 +2199,7 @@
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A31" s="3" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="B31" s="4">
         <v>91732802</v>
@@ -2211,10 +2208,10 @@
         <v>98820079</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F31" s="2" t="s">
         <v>17</v>
@@ -2250,10 +2247,10 @@
         <v>98820081</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="F32" s="2" t="s">
         <v>12</v>
@@ -2280,7 +2277,7 @@
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A33" s="3" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="B33" s="2">
         <v>91546282</v>
@@ -2289,10 +2286,10 @@
         <v>98820079</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F33" s="2" t="s">
         <v>17</v>
@@ -2321,7 +2318,7 @@
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A34" s="3" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="B34" s="2">
         <v>91732791</v>
@@ -2330,10 +2327,10 @@
         <v>98820079</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F34" s="2" t="s">
         <v>17</v>
@@ -2362,7 +2359,7 @@
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A35" s="3" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="B35" s="2">
         <v>91732818</v>
@@ -2371,10 +2368,10 @@
         <v>98820079</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F35" s="2" t="s">
         <v>17</v>
@@ -2403,7 +2400,7 @@
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A36" s="3" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="B36" s="2">
         <v>91732782</v>
@@ -2412,10 +2409,10 @@
         <v>98820079</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F36" s="2" t="s">
         <v>17</v>
@@ -2444,7 +2441,7 @@
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A37" s="3" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="B37" s="2">
         <v>91546307</v>
@@ -2453,10 +2450,10 @@
         <v>98820079</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F37" s="2" t="s">
         <v>17</v>
@@ -2485,7 +2482,7 @@
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A38" s="3" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="B38" s="13">
         <v>91732842</v>
@@ -2494,10 +2491,10 @@
         <v>98820081</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F38" s="2" t="s">
         <v>17</v>
@@ -2526,7 +2523,7 @@
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A39" s="3" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="B39" s="13">
         <v>91732793</v>
@@ -2535,10 +2532,10 @@
         <v>98820081</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F39" s="2" t="s">
         <v>17</v>
@@ -2567,7 +2564,7 @@
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A40" s="3" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="B40" s="13">
         <v>91732840</v>
@@ -2576,10 +2573,10 @@
         <v>98820081</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F40" s="2" t="s">
         <v>17</v>
@@ -2608,7 +2605,7 @@
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A41" s="3" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="B41" s="13">
         <v>91732817</v>
@@ -2617,10 +2614,10 @@
         <v>98820081</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F41" s="2" t="s">
         <v>17</v>
@@ -2649,7 +2646,7 @@
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A42" s="3" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="B42" s="13">
         <v>91732792</v>
@@ -2658,10 +2655,10 @@
         <v>98820081</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F42" s="2" t="s">
         <v>17</v>
@@ -2690,7 +2687,7 @@
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A43" s="3" t="s">
-        <v>133</v>
+        <v>123</v>
       </c>
       <c r="B43" s="13">
         <v>91732796</v>
@@ -2699,10 +2696,10 @@
         <v>98820081</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F43" s="2" t="s">
         <v>17</v>
@@ -2731,7 +2728,7 @@
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A44" s="3" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="B44" s="2">
         <v>91546227</v>
@@ -2740,10 +2737,10 @@
         <v>98820079</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F44" s="2" t="s">
         <v>17</v>
@@ -2772,7 +2769,7 @@
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A45" s="3" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="B45" s="2">
         <v>91732786</v>
@@ -2781,10 +2778,10 @@
         <v>98820079</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F45" s="2" t="s">
         <v>17</v>
@@ -2813,7 +2810,7 @@
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A46" s="3" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="B46" s="2">
         <v>91732808</v>
@@ -2822,10 +2819,10 @@
         <v>98820079</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F46" s="2" t="s">
         <v>17</v>
@@ -2854,7 +2851,7 @@
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A47" s="3" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="B47" s="2">
         <v>91546277</v>
@@ -2863,10 +2860,10 @@
         <v>98820079</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F47" s="2" t="s">
         <v>17</v>
@@ -2895,7 +2892,7 @@
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A48" s="3" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="B48" s="2">
         <v>91732798</v>
@@ -2904,10 +2901,10 @@
         <v>98820079</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F48" s="2" t="s">
         <v>17</v>
@@ -2936,19 +2933,19 @@
     </row>
     <row r="49" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A49" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="B49" s="2">
+        <v>127</v>
+      </c>
+      <c r="B49" s="13">
         <v>91732794</v>
       </c>
       <c r="C49" s="2">
         <v>98820081</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F49" s="2" t="s">
         <v>17</v>
@@ -2956,7 +2953,7 @@
       <c r="G49" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="H49" s="2" t="s">
+      <c r="H49" s="13" t="s">
         <v>36</v>
       </c>
       <c r="I49" s="4">
@@ -2966,28 +2963,30 @@
         <v>46136</v>
       </c>
       <c r="K49" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="L49" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="L49" s="2">
+        <v>4</v>
+      </c>
       <c r="M49" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A50" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="B50" s="2">
+        <v>128</v>
+      </c>
+      <c r="B50" s="13">
         <v>91732774</v>
       </c>
       <c r="C50" s="2">
         <v>98820081</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F50" s="2" t="s">
         <v>17</v>
@@ -2995,7 +2994,7 @@
       <c r="G50" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="H50" s="2" t="s">
+      <c r="H50" s="13" t="s">
         <v>36</v>
       </c>
       <c r="I50" s="4">
@@ -3005,28 +3004,30 @@
         <v>46136</v>
       </c>
       <c r="K50" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="L50" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="L50" s="2">
+        <v>3</v>
+      </c>
       <c r="M50" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A51" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="B51" s="2">
+        <v>126</v>
+      </c>
+      <c r="B51" s="13">
         <v>91732776</v>
       </c>
       <c r="C51" s="2">
         <v>98820081</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F51" s="2" t="s">
         <v>17</v>
@@ -3034,7 +3035,7 @@
       <c r="G51" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="H51" s="2" t="s">
+      <c r="H51" s="13" t="s">
         <v>36</v>
       </c>
       <c r="I51" s="4">
@@ -3044,28 +3045,30 @@
         <v>46136</v>
       </c>
       <c r="K51" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="L51" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="L51" s="2">
+        <v>5</v>
+      </c>
       <c r="M51" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A52" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="B52" s="2">
+        <v>129</v>
+      </c>
+      <c r="B52" s="13">
         <v>91732801</v>
       </c>
       <c r="C52" s="2">
         <v>98820081</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F52" s="2" t="s">
         <v>17</v>
@@ -3073,7 +3076,7 @@
       <c r="G52" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="H52" s="2" t="s">
+      <c r="H52" s="13" t="s">
         <v>36</v>
       </c>
       <c r="I52" s="4">
@@ -3083,28 +3086,30 @@
         <v>46136</v>
       </c>
       <c r="K52" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="L52" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="L52" s="2">
+        <v>2</v>
+      </c>
       <c r="M52" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A53" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="B53" s="2">
+        <v>125</v>
+      </c>
+      <c r="B53" s="13">
         <v>91732784</v>
       </c>
       <c r="C53" s="2">
         <v>98820081</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F53" s="2" t="s">
         <v>17</v>
@@ -3112,7 +3117,7 @@
       <c r="G53" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="H53" s="2" t="s">
+      <c r="H53" s="13" t="s">
         <v>36</v>
       </c>
       <c r="I53" s="4">
@@ -3122,28 +3127,30 @@
         <v>46136</v>
       </c>
       <c r="K53" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="L53" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="L53" s="2">
+        <v>6</v>
+      </c>
       <c r="M53" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A54" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="B54" s="2">
+        <v>130</v>
+      </c>
+      <c r="B54" s="13">
         <v>91732790</v>
       </c>
       <c r="C54" s="2">
         <v>98820081</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F54" s="2" t="s">
         <v>17</v>
@@ -3151,7 +3158,7 @@
       <c r="G54" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="H54" s="2" t="s">
+      <c r="H54" s="13" t="s">
         <v>36</v>
       </c>
       <c r="I54" s="4">
@@ -3161,16 +3168,18 @@
         <v>46136</v>
       </c>
       <c r="K54" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="L54" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="L54" s="2">
+        <v>1</v>
+      </c>
       <c r="M54" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="55" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A55" s="3" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="B55" s="2">
         <v>91546303</v>
@@ -3179,10 +3188,10 @@
         <v>98820079</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F55" s="2" t="s">
         <v>17</v>
@@ -3211,7 +3220,7 @@
     </row>
     <row r="56" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A56" s="3" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="B56" s="2">
         <v>91546278</v>
@@ -3220,10 +3229,10 @@
         <v>98820079</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F56" s="2" t="s">
         <v>17</v>
@@ -3252,7 +3261,7 @@
     </row>
     <row r="57" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A57" s="3" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="B57" s="2">
         <v>91542774</v>
@@ -3261,10 +3270,10 @@
         <v>98820079</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F57" s="2" t="s">
         <v>17</v>
@@ -3293,7 +3302,7 @@
     </row>
     <row r="58" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A58" s="3" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="B58" s="2">
         <v>91732833</v>
@@ -3302,10 +3311,10 @@
         <v>98820079</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F58" s="2" t="s">
         <v>17</v>
@@ -3334,7 +3343,7 @@
     </row>
     <row r="59" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A59" s="3" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="B59" s="2">
         <v>91732778</v>
@@ -3343,10 +3352,10 @@
         <v>98820079</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F59" s="2" t="s">
         <v>17</v>
@@ -3375,19 +3384,19 @@
     </row>
     <row r="60" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A60" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="B60" s="2">
+        <v>133</v>
+      </c>
+      <c r="B60" s="13">
         <v>91546300</v>
       </c>
       <c r="C60" s="2">
         <v>98820081</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F60" s="2" t="s">
         <v>17</v>
@@ -3395,7 +3404,7 @@
       <c r="G60" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H60" s="2" t="s">
+      <c r="H60" s="13" t="s">
         <v>21</v>
       </c>
       <c r="I60" s="4">
@@ -3405,28 +3414,30 @@
         <v>46136</v>
       </c>
       <c r="K60" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="L60" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="L60" s="2">
+        <v>3</v>
+      </c>
       <c r="M60" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="61" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A61" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="B61" s="2">
+        <v>132</v>
+      </c>
+      <c r="B61" s="13">
         <v>91732839</v>
       </c>
       <c r="C61" s="2">
         <v>98820081</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F61" s="2" t="s">
         <v>17</v>
@@ -3434,7 +3445,7 @@
       <c r="G61" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="H61" s="2" t="s">
+      <c r="H61" s="13" t="s">
         <v>21</v>
       </c>
       <c r="I61" s="4">
@@ -3444,28 +3455,30 @@
         <v>46136</v>
       </c>
       <c r="K61" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="L61" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="L61" s="2">
+        <v>2</v>
+      </c>
       <c r="M61" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="62" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A62" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B62" s="2">
+        <v>134</v>
+      </c>
+      <c r="B62" s="13">
         <v>91546308</v>
       </c>
       <c r="C62" s="2">
         <v>98820081</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F62" s="2" t="s">
         <v>17</v>
@@ -3473,7 +3486,7 @@
       <c r="G62" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="H62" s="2" t="s">
+      <c r="H62" s="13" t="s">
         <v>21</v>
       </c>
       <c r="I62" s="4">
@@ -3483,28 +3496,30 @@
         <v>46136</v>
       </c>
       <c r="K62" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="L62" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="L62" s="2">
+        <v>4</v>
+      </c>
       <c r="M62" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A63" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="B63" s="2">
+        <v>131</v>
+      </c>
+      <c r="B63" s="13">
         <v>91732813</v>
       </c>
       <c r="C63" s="2">
         <v>98820081</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F63" s="2" t="s">
         <v>17</v>
@@ -3512,7 +3527,7 @@
       <c r="G63" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H63" s="2" t="s">
+      <c r="H63" s="13" t="s">
         <v>21</v>
       </c>
       <c r="I63" s="4">
@@ -3522,16 +3537,18 @@
         <v>46136</v>
       </c>
       <c r="K63" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="L63" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="L63" s="2">
+        <v>1</v>
+      </c>
       <c r="M63" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A64" s="3" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="B64" s="13">
         <v>91732804</v>
@@ -3540,10 +3557,10 @@
         <v>98820079</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F64" s="2" t="s">
         <v>17</v>
@@ -3572,7 +3589,7 @@
     </row>
     <row r="65" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A65" s="3" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="B65" s="13">
         <v>91546301</v>
@@ -3581,10 +3598,10 @@
         <v>98820079</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F65" s="2" t="s">
         <v>17</v>
@@ -3613,7 +3630,7 @@
     </row>
     <row r="66" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A66" s="3" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="B66" s="13">
         <v>91732807</v>
@@ -3622,10 +3639,10 @@
         <v>98820079</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F66" s="2" t="s">
         <v>17</v>
@@ -3654,7 +3671,7 @@
     </row>
     <row r="67" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A67" s="3" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="B67" s="13">
         <v>91546332</v>
@@ -3663,10 +3680,10 @@
         <v>98820079</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F67" s="2" t="s">
         <v>17</v>
@@ -3695,7 +3712,7 @@
     </row>
     <row r="68" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A68" s="3" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B68" s="13">
         <v>91546306</v>
@@ -3704,10 +3721,10 @@
         <v>98820079</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F68" s="2" t="s">
         <v>17</v>
@@ -3736,7 +3753,7 @@
     </row>
     <row r="69" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A69" s="3" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B69" s="13">
         <v>91732811</v>
@@ -3745,10 +3762,10 @@
         <v>98820079</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F69" s="2" t="s">
         <v>17</v>
@@ -3786,10 +3803,10 @@
         <v>98820081</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F70" s="2" t="s">
         <v>17</v>
@@ -3825,10 +3842,10 @@
         <v>98820081</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F71" s="2" t="s">
         <v>17</v>
@@ -3864,10 +3881,10 @@
         <v>98820081</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F72" s="2" t="s">
         <v>17</v>
@@ -3903,10 +3920,10 @@
         <v>98820081</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F73" s="2" t="s">
         <v>17</v>
@@ -3933,7 +3950,7 @@
     </row>
     <row r="74" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A74" s="3" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="B74" s="12">
         <v>91546258</v>
@@ -3942,10 +3959,10 @@
         <v>98820079</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F74" s="2" t="s">
         <v>17</v>
@@ -3974,7 +3991,7 @@
     </row>
     <row r="75" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A75" s="3" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="B75" s="12">
         <v>91732783</v>
@@ -3983,10 +4000,10 @@
         <v>98820079</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F75" s="2" t="s">
         <v>17</v>
@@ -4015,7 +4032,7 @@
     </row>
     <row r="76" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A76" s="3" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="B76" s="12">
         <v>91732779</v>
@@ -4024,10 +4041,10 @@
         <v>98820079</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F76" s="2" t="s">
         <v>17</v>
@@ -4056,7 +4073,7 @@
     </row>
     <row r="77" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A77" s="3" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="B77" s="12">
         <v>91732789</v>
@@ -4065,10 +4082,10 @@
         <v>98820079</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F77" s="2" t="s">
         <v>17</v>
@@ -4097,7 +4114,7 @@
     </row>
     <row r="78" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A78" s="3" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="B78" s="12">
         <v>91546253</v>
@@ -4106,10 +4123,10 @@
         <v>98820079</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E78" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F78" s="2" t="s">
         <v>17</v>
@@ -4138,7 +4155,7 @@
     </row>
     <row r="79" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A79" s="3" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="B79" s="13">
         <v>91732816</v>
@@ -4147,10 +4164,10 @@
         <v>98820079</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F79" s="2" t="s">
         <v>17</v>
@@ -4179,7 +4196,7 @@
     </row>
     <row r="80" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A80" s="3" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="B80" s="13">
         <v>91546325</v>
@@ -4188,10 +4205,10 @@
         <v>98820079</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F80" s="2" t="s">
         <v>17</v>
@@ -4220,7 +4237,7 @@
     </row>
     <row r="81" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A81" s="3" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="B81" s="13">
         <v>91732805</v>
@@ -4229,10 +4246,10 @@
         <v>98820079</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F81" s="2" t="s">
         <v>17</v>
@@ -4261,7 +4278,7 @@
     </row>
     <row r="82" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A82" s="3" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="B82" s="13">
         <v>91732800</v>
@@ -4270,10 +4287,10 @@
         <v>98820079</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E82" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F82" s="2" t="s">
         <v>17</v>
@@ -4311,10 +4328,10 @@
         <v>98820079</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="F83" s="2" t="s">
         <v>15</v>
@@ -4350,10 +4367,10 @@
         <v>98820079</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="F84" s="2" t="s">
         <v>12</v>
@@ -4389,10 +4406,10 @@
         <v>4</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="F85" s="2" t="s">
         <v>35</v>
@@ -4428,10 +4445,10 @@
         <v>4</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="F86" s="2" t="s">
         <v>35</v>
@@ -4467,10 +4484,10 @@
         <v>4</v>
       </c>
       <c r="D87" s="3" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="E87" s="3" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="F87" s="2" t="s">
         <v>39</v>

</xml_diff>

<commit_message>
Stand renaming and AMR installs
</commit_message>
<xml_diff>
--- a/EVG_Lake_Michelle_Meter_Hierarchy_2026-07-03.xlsx
+++ b/EVG_Lake_Michelle_Meter_Hierarchy_2026-07-03.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://voltano-my.sharepoint.com/personal/ruan_vh_voltano_com/Documents/Desktop/Voltano/Clients/Evergreen/Lake Michelle Noordhoek/Site Management/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="570" documentId="8_{E5281369-C957-4F01-BD7F-34BF193967CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F5D8F626-F6F8-4F6C-8C6D-46B66EFA8383}"/>
+  <xr:revisionPtr revIDLastSave="643" documentId="8_{E5281369-C957-4F01-BD7F-34BF193967CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2B5F2B9B-1969-4B1B-9C53-BFD42DB28BFE}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{AE166FFD-83CC-4E71-A293-C6082B1A6C83}"/>
   </bookViews>
@@ -164,18 +164,6 @@
     <t>3x800A</t>
   </si>
   <si>
-    <t>001</t>
-  </si>
-  <si>
-    <t>002</t>
-  </si>
-  <si>
-    <t>003</t>
-  </si>
-  <si>
-    <t>004</t>
-  </si>
-  <si>
     <t>036</t>
   </si>
   <si>
@@ -194,51 +182,6 @@
     <t>050</t>
   </si>
   <si>
-    <t>057</t>
-  </si>
-  <si>
-    <t>059</t>
-  </si>
-  <si>
-    <t>060</t>
-  </si>
-  <si>
-    <t>061</t>
-  </si>
-  <si>
-    <t>062</t>
-  </si>
-  <si>
-    <t>063</t>
-  </si>
-  <si>
-    <t>064</t>
-  </si>
-  <si>
-    <t>065</t>
-  </si>
-  <si>
-    <t>066</t>
-  </si>
-  <si>
-    <t>067</t>
-  </si>
-  <si>
-    <t>068</t>
-  </si>
-  <si>
-    <t>069</t>
-  </si>
-  <si>
-    <t>070</t>
-  </si>
-  <si>
-    <t>071</t>
-  </si>
-  <si>
-    <t>072</t>
-  </si>
-  <si>
     <t>073</t>
   </si>
   <si>
@@ -447,6 +390,63 @@
   </si>
   <si>
     <t>70</t>
+  </si>
+  <si>
+    <t>68</t>
+  </si>
+  <si>
+    <t>67</t>
+  </si>
+  <si>
+    <t>66</t>
+  </si>
+  <si>
+    <t>65</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>38</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>39</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>40</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>41</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>42</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>43</t>
+  </si>
+  <si>
+    <t>11</t>
   </si>
 </sst>
 </file>
@@ -547,7 +547,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -591,6 +591,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -989,13 +992,13 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>73</v>
+        <v>54</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>76</v>
+        <v>57</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>5</v>
@@ -1004,27 +1007,27 @@
         <v>2</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>85</v>
+        <v>66</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>84</v>
+        <v>65</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>83</v>
+        <v>64</v>
       </c>
       <c r="K1" s="10" t="s">
-        <v>82</v>
+        <v>63</v>
       </c>
       <c r="L1" s="10" t="s">
-        <v>86</v>
+        <v>67</v>
       </c>
       <c r="M1" s="10" t="s">
-        <v>124</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A2" s="3" t="s">
-        <v>98</v>
+        <v>79</v>
       </c>
       <c r="B2" s="13">
         <v>91732777</v>
@@ -1033,10 +1036,10 @@
         <v>98820079</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>17</v>
@@ -1065,7 +1068,7 @@
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
-        <v>97</v>
+        <v>78</v>
       </c>
       <c r="B3" s="13">
         <v>91732837</v>
@@ -1074,10 +1077,10 @@
         <v>98820079</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>17</v>
@@ -1106,7 +1109,7 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="B4" s="13">
         <v>91733081</v>
@@ -1115,10 +1118,10 @@
         <v>98820079</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>17</v>
@@ -1147,7 +1150,7 @@
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A5" s="3" t="s">
-        <v>99</v>
+        <v>80</v>
       </c>
       <c r="B5" s="13">
         <v>91732799</v>
@@ -1156,10 +1159,10 @@
         <v>98820079</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>17</v>
@@ -1188,7 +1191,7 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A6" s="3" t="s">
-        <v>100</v>
+        <v>81</v>
       </c>
       <c r="B6" s="13">
         <v>91546302</v>
@@ -1197,10 +1200,10 @@
         <v>98820079</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>17</v>
@@ -1229,7 +1232,7 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A7" s="3" t="s">
-        <v>101</v>
+        <v>82</v>
       </c>
       <c r="B7" s="13">
         <v>91732803</v>
@@ -1238,10 +1241,10 @@
         <v>98820079</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>17</v>
@@ -1270,7 +1273,7 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A8" s="3" t="s">
-        <v>103</v>
+        <v>84</v>
       </c>
       <c r="B8" s="13">
         <v>91546328</v>
@@ -1279,10 +1282,10 @@
         <v>98820079</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>17</v>
@@ -1311,7 +1314,7 @@
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A9" s="3" t="s">
-        <v>104</v>
+        <v>85</v>
       </c>
       <c r="B9" s="13">
         <v>91546327</v>
@@ -1320,10 +1323,10 @@
         <v>98820079</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>17</v>
@@ -1352,7 +1355,7 @@
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A10" s="3" t="s">
-        <v>102</v>
+        <v>83</v>
       </c>
       <c r="B10" s="13">
         <v>91546252</v>
@@ -1361,10 +1364,10 @@
         <v>98820079</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>17</v>
@@ -1393,7 +1396,7 @@
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A11" s="3" t="s">
-        <v>105</v>
+        <v>86</v>
       </c>
       <c r="B11" s="13">
         <v>91732812</v>
@@ -1402,10 +1405,10 @@
         <v>98820079</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>17</v>
@@ -1434,7 +1437,7 @@
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A12" s="3" t="s">
-        <v>106</v>
+        <v>87</v>
       </c>
       <c r="B12" s="13">
         <v>91546326</v>
@@ -1443,10 +1446,10 @@
         <v>98820079</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>17</v>
@@ -1475,7 +1478,7 @@
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A13" s="3" t="s">
-        <v>107</v>
+        <v>88</v>
       </c>
       <c r="B13" s="13">
         <v>91732785</v>
@@ -1484,10 +1487,10 @@
         <v>98820079</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>17</v>
@@ -1516,7 +1519,7 @@
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A14" s="3" t="s">
-        <v>111</v>
+        <v>92</v>
       </c>
       <c r="B14" s="13">
         <v>91732797</v>
@@ -1525,10 +1528,10 @@
         <v>98820081</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>17</v>
@@ -1557,7 +1560,7 @@
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A15" s="3" t="s">
-        <v>110</v>
+        <v>91</v>
       </c>
       <c r="B15" s="13">
         <v>91732835</v>
@@ -1566,10 +1569,10 @@
         <v>98820081</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>17</v>
@@ -1598,7 +1601,7 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A16" s="3" t="s">
-        <v>109</v>
+        <v>90</v>
       </c>
       <c r="B16" s="13">
         <v>91546283</v>
@@ -1607,10 +1610,10 @@
         <v>98820081</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>17</v>
@@ -1639,7 +1642,7 @@
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A17" s="3" t="s">
-        <v>108</v>
+        <v>89</v>
       </c>
       <c r="B17" s="13">
         <v>91732806</v>
@@ -1648,10 +1651,10 @@
         <v>98820081</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>17</v>
@@ -1680,7 +1683,7 @@
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A18" s="3" t="s">
-        <v>112</v>
+        <v>93</v>
       </c>
       <c r="B18" s="13">
         <v>91732775</v>
@@ -1689,10 +1692,10 @@
         <v>98820081</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>17</v>
@@ -1721,7 +1724,7 @@
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A19" s="3" t="s">
-        <v>69</v>
+        <v>50</v>
       </c>
       <c r="B19" s="2">
         <v>91732809</v>
@@ -1730,10 +1733,10 @@
         <v>98820079</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>17</v>
@@ -1760,7 +1763,7 @@
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A20" s="3" t="s">
-        <v>70</v>
+        <v>51</v>
       </c>
       <c r="B20" s="2">
         <v>91732788</v>
@@ -1769,10 +1772,10 @@
         <v>98820079</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>17</v>
@@ -1799,7 +1802,7 @@
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A21" s="3" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="B21" s="2">
         <v>91546333</v>
@@ -1808,10 +1811,10 @@
         <v>98820079</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>17</v>
@@ -1838,7 +1841,7 @@
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A22" s="3" t="s">
-        <v>72</v>
+        <v>53</v>
       </c>
       <c r="B22" s="2">
         <v>91732814</v>
@@ -1847,10 +1850,10 @@
         <v>98820079</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>17</v>
@@ -1877,7 +1880,7 @@
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A23" s="3" t="s">
-        <v>116</v>
+        <v>97</v>
       </c>
       <c r="B23" s="13">
         <v>91732831</v>
@@ -1886,10 +1889,10 @@
         <v>98820081</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F23" s="2" t="s">
         <v>17</v>
@@ -1918,7 +1921,7 @@
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A24" s="3" t="s">
-        <v>115</v>
+        <v>96</v>
       </c>
       <c r="B24" s="13">
         <v>91732781</v>
@@ -1927,10 +1930,10 @@
         <v>98820081</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>17</v>
@@ -1959,7 +1962,7 @@
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A25" s="3" t="s">
-        <v>117</v>
+        <v>98</v>
       </c>
       <c r="B25" s="13">
         <v>91732815</v>
@@ -1968,10 +1971,10 @@
         <v>98820081</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>17</v>
@@ -2000,7 +2003,7 @@
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A26" s="3" t="s">
-        <v>114</v>
+        <v>95</v>
       </c>
       <c r="B26" s="13">
         <v>91732780</v>
@@ -2009,10 +2012,10 @@
         <v>98820081</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F26" s="2" t="s">
         <v>17</v>
@@ -2041,7 +2044,7 @@
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A27" s="3" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="B27" s="13">
         <v>91732841</v>
@@ -2050,10 +2053,10 @@
         <v>98820081</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F27" s="2" t="s">
         <v>17</v>
@@ -2082,7 +2085,7 @@
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A28" s="3" t="s">
-        <v>65</v>
+        <v>46</v>
       </c>
       <c r="B28" s="4">
         <v>91732795</v>
@@ -2091,10 +2094,10 @@
         <v>98820079</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F28" s="2" t="s">
         <v>17</v>
@@ -2121,7 +2124,7 @@
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A29" s="3" t="s">
-        <v>66</v>
+        <v>47</v>
       </c>
       <c r="B29" s="4">
         <v>91546331</v>
@@ -2130,10 +2133,10 @@
         <v>98820079</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F29" s="2" t="s">
         <v>17</v>
@@ -2160,7 +2163,7 @@
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A30" s="3" t="s">
-        <v>67</v>
+        <v>48</v>
       </c>
       <c r="B30" s="4">
         <v>91732836</v>
@@ -2169,10 +2172,10 @@
         <v>98820079</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F30" s="2" t="s">
         <v>17</v>
@@ -2199,7 +2202,7 @@
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A31" s="3" t="s">
-        <v>68</v>
+        <v>49</v>
       </c>
       <c r="B31" s="4">
         <v>91732802</v>
@@ -2208,10 +2211,10 @@
         <v>98820079</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F31" s="2" t="s">
         <v>17</v>
@@ -2240,17 +2243,17 @@
       <c r="A32" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B32" s="2">
+      <c r="B32" s="13">
         <v>90151406</v>
       </c>
       <c r="C32" s="2">
         <v>98820081</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>78</v>
+        <v>59</v>
       </c>
       <c r="F32" s="2" t="s">
         <v>12</v>
@@ -2258,7 +2261,7 @@
       <c r="G32" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H32" s="2" t="s">
+      <c r="H32" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I32" s="4">
@@ -2268,28 +2271,30 @@
         <v>46162</v>
       </c>
       <c r="K32" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="L32" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="L32" s="2">
+        <v>1</v>
+      </c>
       <c r="M32" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A33" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="B33" s="2">
+        <v>120</v>
+      </c>
+      <c r="B33" s="13">
         <v>91546282</v>
       </c>
       <c r="C33" s="2">
         <v>98820079</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F33" s="2" t="s">
         <v>17</v>
@@ -2297,7 +2302,7 @@
       <c r="G33" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H33" s="2" t="s">
+      <c r="H33" s="13" t="s">
         <v>30</v>
       </c>
       <c r="I33" s="4">
@@ -2313,24 +2318,24 @@
         <v>1</v>
       </c>
       <c r="M33" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A34" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="B34" s="2">
+        <v>121</v>
+      </c>
+      <c r="B34" s="13">
         <v>91732791</v>
       </c>
       <c r="C34" s="2">
         <v>98820079</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F34" s="2" t="s">
         <v>17</v>
@@ -2338,7 +2343,7 @@
       <c r="G34" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="H34" s="2" t="s">
+      <c r="H34" s="13" t="s">
         <v>30</v>
       </c>
       <c r="I34" s="4">
@@ -2354,24 +2359,24 @@
         <v>2</v>
       </c>
       <c r="M34" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A35" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="B35" s="2">
+        <v>122</v>
+      </c>
+      <c r="B35" s="13">
         <v>91732818</v>
       </c>
       <c r="C35" s="2">
         <v>98820079</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F35" s="2" t="s">
         <v>17</v>
@@ -2379,7 +2384,7 @@
       <c r="G35" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="H35" s="2" t="s">
+      <c r="H35" s="13" t="s">
         <v>30</v>
       </c>
       <c r="I35" s="4">
@@ -2395,24 +2400,24 @@
         <v>3</v>
       </c>
       <c r="M35" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A36" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="B36" s="2">
+        <v>123</v>
+      </c>
+      <c r="B36" s="13">
         <v>91732782</v>
       </c>
       <c r="C36" s="2">
         <v>98820079</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F36" s="2" t="s">
         <v>17</v>
@@ -2420,7 +2425,7 @@
       <c r="G36" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="H36" s="2" t="s">
+      <c r="H36" s="13" t="s">
         <v>30</v>
       </c>
       <c r="I36" s="4">
@@ -2436,24 +2441,24 @@
         <v>4</v>
       </c>
       <c r="M36" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A37" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="B37" s="2">
+        <v>124</v>
+      </c>
+      <c r="B37" s="13">
         <v>91546307</v>
       </c>
       <c r="C37" s="2">
         <v>98820079</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F37" s="2" t="s">
         <v>17</v>
@@ -2461,7 +2466,7 @@
       <c r="G37" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="H37" s="2" t="s">
+      <c r="H37" s="13" t="s">
         <v>30</v>
       </c>
       <c r="I37" s="4">
@@ -2477,12 +2482,12 @@
         <v>5</v>
       </c>
       <c r="M37" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A38" s="3" t="s">
-        <v>120</v>
+        <v>101</v>
       </c>
       <c r="B38" s="13">
         <v>91732842</v>
@@ -2491,10 +2496,10 @@
         <v>98820081</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F38" s="2" t="s">
         <v>17</v>
@@ -2523,7 +2528,7 @@
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A39" s="3" t="s">
-        <v>119</v>
+        <v>100</v>
       </c>
       <c r="B39" s="13">
         <v>91732793</v>
@@ -2532,10 +2537,10 @@
         <v>98820081</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F39" s="2" t="s">
         <v>17</v>
@@ -2564,7 +2569,7 @@
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A40" s="3" t="s">
-        <v>121</v>
+        <v>102</v>
       </c>
       <c r="B40" s="13">
         <v>91732840</v>
@@ -2573,10 +2578,10 @@
         <v>98820081</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F40" s="2" t="s">
         <v>17</v>
@@ -2605,7 +2610,7 @@
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A41" s="3" t="s">
-        <v>118</v>
+        <v>99</v>
       </c>
       <c r="B41" s="13">
         <v>91732817</v>
@@ -2614,10 +2619,10 @@
         <v>98820081</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F41" s="2" t="s">
         <v>17</v>
@@ -2646,7 +2651,7 @@
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A42" s="3" t="s">
-        <v>122</v>
+        <v>103</v>
       </c>
       <c r="B42" s="13">
         <v>91732792</v>
@@ -2655,10 +2660,10 @@
         <v>98820081</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F42" s="2" t="s">
         <v>17</v>
@@ -2687,7 +2692,7 @@
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A43" s="3" t="s">
-        <v>123</v>
+        <v>104</v>
       </c>
       <c r="B43" s="13">
         <v>91732796</v>
@@ -2696,10 +2701,10 @@
         <v>98820081</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F43" s="2" t="s">
         <v>17</v>
@@ -2728,19 +2733,19 @@
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A44" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="B44" s="2">
+        <v>125</v>
+      </c>
+      <c r="B44" s="13">
         <v>91546227</v>
       </c>
       <c r="C44" s="2">
         <v>98820079</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F44" s="2" t="s">
         <v>17</v>
@@ -2748,7 +2753,7 @@
       <c r="G44" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="H44" s="2" t="s">
+      <c r="H44" s="13" t="s">
         <v>31</v>
       </c>
       <c r="I44" s="4">
@@ -2764,24 +2769,24 @@
         <v>1</v>
       </c>
       <c r="M44" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A45" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="B45" s="2">
+        <v>126</v>
+      </c>
+      <c r="B45" s="13">
         <v>91732786</v>
       </c>
       <c r="C45" s="2">
         <v>98820079</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F45" s="2" t="s">
         <v>17</v>
@@ -2789,7 +2794,7 @@
       <c r="G45" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="H45" s="2" t="s">
+      <c r="H45" s="13" t="s">
         <v>31</v>
       </c>
       <c r="I45" s="4">
@@ -2805,24 +2810,24 @@
         <v>2</v>
       </c>
       <c r="M45" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A46" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="B46" s="2">
+        <v>127</v>
+      </c>
+      <c r="B46" s="13">
         <v>91732808</v>
       </c>
       <c r="C46" s="2">
         <v>98820079</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F46" s="2" t="s">
         <v>17</v>
@@ -2830,7 +2835,7 @@
       <c r="G46" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="H46" s="2" t="s">
+      <c r="H46" s="13" t="s">
         <v>31</v>
       </c>
       <c r="I46" s="4">
@@ -2846,24 +2851,24 @@
         <v>3</v>
       </c>
       <c r="M46" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A47" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="B47" s="2">
+        <v>128</v>
+      </c>
+      <c r="B47" s="13">
         <v>91546277</v>
       </c>
       <c r="C47" s="2">
         <v>98820079</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F47" s="2" t="s">
         <v>17</v>
@@ -2871,7 +2876,7 @@
       <c r="G47" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="H47" s="2" t="s">
+      <c r="H47" s="13" t="s">
         <v>31</v>
       </c>
       <c r="I47" s="4">
@@ -2887,24 +2892,24 @@
         <v>4</v>
       </c>
       <c r="M47" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A48" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="B48" s="2">
+        <v>129</v>
+      </c>
+      <c r="B48" s="13">
         <v>91732798</v>
       </c>
       <c r="C48" s="2">
         <v>98820079</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F48" s="2" t="s">
         <v>17</v>
@@ -2912,7 +2917,7 @@
       <c r="G48" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="H48" s="2" t="s">
+      <c r="H48" s="13" t="s">
         <v>31</v>
       </c>
       <c r="I48" s="4">
@@ -2928,12 +2933,12 @@
         <v>5</v>
       </c>
       <c r="M48" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A49" s="3" t="s">
-        <v>127</v>
+        <v>108</v>
       </c>
       <c r="B49" s="13">
         <v>91732794</v>
@@ -2942,10 +2947,10 @@
         <v>98820081</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F49" s="2" t="s">
         <v>17</v>
@@ -2974,7 +2979,7 @@
     </row>
     <row r="50" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A50" s="3" t="s">
-        <v>128</v>
+        <v>109</v>
       </c>
       <c r="B50" s="13">
         <v>91732774</v>
@@ -2983,10 +2988,10 @@
         <v>98820081</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F50" s="2" t="s">
         <v>17</v>
@@ -3015,7 +3020,7 @@
     </row>
     <row r="51" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A51" s="3" t="s">
-        <v>126</v>
+        <v>107</v>
       </c>
       <c r="B51" s="13">
         <v>91732776</v>
@@ -3024,10 +3029,10 @@
         <v>98820081</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F51" s="2" t="s">
         <v>17</v>
@@ -3056,7 +3061,7 @@
     </row>
     <row r="52" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A52" s="3" t="s">
-        <v>129</v>
+        <v>110</v>
       </c>
       <c r="B52" s="13">
         <v>91732801</v>
@@ -3065,10 +3070,10 @@
         <v>98820081</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F52" s="2" t="s">
         <v>17</v>
@@ -3097,7 +3102,7 @@
     </row>
     <row r="53" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A53" s="3" t="s">
-        <v>125</v>
+        <v>106</v>
       </c>
       <c r="B53" s="13">
         <v>91732784</v>
@@ -3106,10 +3111,10 @@
         <v>98820081</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F53" s="2" t="s">
         <v>17</v>
@@ -3138,7 +3143,7 @@
     </row>
     <row r="54" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A54" s="3" t="s">
-        <v>130</v>
+        <v>111</v>
       </c>
       <c r="B54" s="13">
         <v>91732790</v>
@@ -3147,10 +3152,10 @@
         <v>98820081</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F54" s="2" t="s">
         <v>17</v>
@@ -3179,19 +3184,19 @@
     </row>
     <row r="55" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A55" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="B55" s="2">
+        <v>134</v>
+      </c>
+      <c r="B55" s="13">
         <v>91546303</v>
       </c>
       <c r="C55" s="2">
         <v>98820079</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F55" s="2" t="s">
         <v>17</v>
@@ -3199,7 +3204,7 @@
       <c r="G55" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="H55" s="2" t="s">
+      <c r="H55" s="13" t="s">
         <v>32</v>
       </c>
       <c r="I55" s="4">
@@ -3215,24 +3220,24 @@
         <v>1</v>
       </c>
       <c r="M55" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A56" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="B56" s="2">
+        <v>133</v>
+      </c>
+      <c r="B56" s="13">
         <v>91546278</v>
       </c>
       <c r="C56" s="2">
         <v>98820079</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F56" s="2" t="s">
         <v>17</v>
@@ -3240,7 +3245,7 @@
       <c r="G56" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="H56" s="2" t="s">
+      <c r="H56" s="13" t="s">
         <v>32</v>
       </c>
       <c r="I56" s="4">
@@ -3256,24 +3261,24 @@
         <v>2</v>
       </c>
       <c r="M56" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="57" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A57" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="B57" s="2">
+        <v>131</v>
+      </c>
+      <c r="B57" s="13">
         <v>91542774</v>
       </c>
       <c r="C57" s="2">
         <v>98820079</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F57" s="2" t="s">
         <v>17</v>
@@ -3281,7 +3286,7 @@
       <c r="G57" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="H57" s="2" t="s">
+      <c r="H57" s="13" t="s">
         <v>32</v>
       </c>
       <c r="I57" s="4">
@@ -3297,24 +3302,24 @@
         <v>3</v>
       </c>
       <c r="M57" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A58" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="B58" s="2">
+        <v>132</v>
+      </c>
+      <c r="B58" s="13">
         <v>91732833</v>
       </c>
       <c r="C58" s="2">
         <v>98820079</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F58" s="2" t="s">
         <v>17</v>
@@ -3322,7 +3327,7 @@
       <c r="G58" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="H58" s="2" t="s">
+      <c r="H58" s="13" t="s">
         <v>32</v>
       </c>
       <c r="I58" s="4">
@@ -3338,24 +3343,24 @@
         <v>4</v>
       </c>
       <c r="M58" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A59" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="B59" s="2">
+        <v>130</v>
+      </c>
+      <c r="B59" s="13">
         <v>91732778</v>
       </c>
       <c r="C59" s="2">
         <v>98820079</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F59" s="2" t="s">
         <v>17</v>
@@ -3363,7 +3368,7 @@
       <c r="G59" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="H59" s="2" t="s">
+      <c r="H59" s="13" t="s">
         <v>32</v>
       </c>
       <c r="I59" s="4">
@@ -3379,12 +3384,12 @@
         <v>5</v>
       </c>
       <c r="M59" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="60" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A60" s="3" t="s">
-        <v>133</v>
+        <v>114</v>
       </c>
       <c r="B60" s="13">
         <v>91546300</v>
@@ -3393,10 +3398,10 @@
         <v>98820081</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F60" s="2" t="s">
         <v>17</v>
@@ -3425,7 +3430,7 @@
     </row>
     <row r="61" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A61" s="3" t="s">
-        <v>132</v>
+        <v>113</v>
       </c>
       <c r="B61" s="13">
         <v>91732839</v>
@@ -3434,10 +3439,10 @@
         <v>98820081</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F61" s="2" t="s">
         <v>17</v>
@@ -3466,7 +3471,7 @@
     </row>
     <row r="62" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A62" s="3" t="s">
-        <v>134</v>
+        <v>115</v>
       </c>
       <c r="B62" s="13">
         <v>91546308</v>
@@ -3475,10 +3480,10 @@
         <v>98820081</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F62" s="2" t="s">
         <v>17</v>
@@ -3507,7 +3512,7 @@
     </row>
     <row r="63" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A63" s="3" t="s">
-        <v>131</v>
+        <v>112</v>
       </c>
       <c r="B63" s="13">
         <v>91732813</v>
@@ -3516,10 +3521,10 @@
         <v>98820081</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F63" s="2" t="s">
         <v>17</v>
@@ -3548,7 +3553,7 @@
     </row>
     <row r="64" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A64" s="3" t="s">
-        <v>90</v>
+        <v>71</v>
       </c>
       <c r="B64" s="13">
         <v>91732804</v>
@@ -3557,10 +3562,10 @@
         <v>98820079</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F64" s="2" t="s">
         <v>17</v>
@@ -3589,7 +3594,7 @@
     </row>
     <row r="65" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A65" s="3" t="s">
-        <v>91</v>
+        <v>72</v>
       </c>
       <c r="B65" s="13">
         <v>91546301</v>
@@ -3598,10 +3603,10 @@
         <v>98820079</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F65" s="2" t="s">
         <v>17</v>
@@ -3630,7 +3635,7 @@
     </row>
     <row r="66" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A66" s="3" t="s">
-        <v>92</v>
+        <v>73</v>
       </c>
       <c r="B66" s="13">
         <v>91732807</v>
@@ -3639,10 +3644,10 @@
         <v>98820079</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F66" s="2" t="s">
         <v>17</v>
@@ -3671,7 +3676,7 @@
     </row>
     <row r="67" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A67" s="3" t="s">
-        <v>89</v>
+        <v>70</v>
       </c>
       <c r="B67" s="13">
         <v>91546332</v>
@@ -3680,10 +3685,10 @@
         <v>98820079</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F67" s="2" t="s">
         <v>17</v>
@@ -3712,7 +3717,7 @@
     </row>
     <row r="68" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A68" s="3" t="s">
-        <v>88</v>
+        <v>69</v>
       </c>
       <c r="B68" s="13">
         <v>91546306</v>
@@ -3721,10 +3726,10 @@
         <v>98820079</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F68" s="2" t="s">
         <v>17</v>
@@ -3753,7 +3758,7 @@
     </row>
     <row r="69" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A69" s="3" t="s">
-        <v>87</v>
+        <v>68</v>
       </c>
       <c r="B69" s="13">
         <v>91732811</v>
@@ -3762,10 +3767,10 @@
         <v>98820079</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F69" s="2" t="s">
         <v>17</v>
@@ -3794,19 +3799,19 @@
     </row>
     <row r="70" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A70" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="B70" s="2">
+        <v>117</v>
+      </c>
+      <c r="B70" s="13">
         <v>91732773</v>
       </c>
       <c r="C70" s="2">
         <v>98820081</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F70" s="2" t="s">
         <v>17</v>
@@ -3814,7 +3819,7 @@
       <c r="G70" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="H70" s="2" t="s">
+      <c r="H70" s="13" t="s">
         <v>16</v>
       </c>
       <c r="I70" s="4">
@@ -3824,28 +3829,30 @@
         <v>46136</v>
       </c>
       <c r="K70" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="L70" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="L70" s="2">
+        <v>3</v>
+      </c>
       <c r="M70" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="71" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A71" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="B71" s="2">
+        <v>118</v>
+      </c>
+      <c r="B71" s="13">
         <v>91732810</v>
       </c>
       <c r="C71" s="2">
         <v>98820081</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F71" s="2" t="s">
         <v>17</v>
@@ -3853,7 +3860,7 @@
       <c r="G71" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="H71" s="2" t="s">
+      <c r="H71" s="13" t="s">
         <v>16</v>
       </c>
       <c r="I71" s="4">
@@ -3863,28 +3870,30 @@
         <v>46136</v>
       </c>
       <c r="K71" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="L71" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="L71" s="2">
+        <v>2</v>
+      </c>
       <c r="M71" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="72" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A72" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="B72" s="2">
+        <v>116</v>
+      </c>
+      <c r="B72" s="13">
         <v>91732787</v>
       </c>
       <c r="C72" s="2">
         <v>98820081</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F72" s="2" t="s">
         <v>17</v>
@@ -3892,7 +3901,7 @@
       <c r="G72" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="H72" s="2" t="s">
+      <c r="H72" s="13" t="s">
         <v>16</v>
       </c>
       <c r="I72" s="4">
@@ -3902,28 +3911,30 @@
         <v>46136</v>
       </c>
       <c r="K72" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="L72" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="L72" s="2">
+        <v>4</v>
+      </c>
       <c r="M72" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="73" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A73" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="B73" s="2">
+        <v>119</v>
+      </c>
+      <c r="B73" s="13">
         <v>91732771</v>
       </c>
       <c r="C73" s="2">
         <v>98820081</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F73" s="2" t="s">
         <v>17</v>
@@ -3931,7 +3942,7 @@
       <c r="G73" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="H73" s="2" t="s">
+      <c r="H73" s="13" t="s">
         <v>16</v>
       </c>
       <c r="I73" s="4">
@@ -3941,16 +3952,18 @@
         <v>46136</v>
       </c>
       <c r="K73" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="L73" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="L73" s="2">
+        <v>1</v>
+      </c>
       <c r="M73" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="74" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A74" s="3" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B74" s="12">
         <v>91546258</v>
@@ -3959,10 +3972,10 @@
         <v>98820079</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F74" s="2" t="s">
         <v>17</v>
@@ -3991,7 +4004,7 @@
     </row>
     <row r="75" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A75" s="3" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="B75" s="12">
         <v>91732783</v>
@@ -4000,10 +4013,10 @@
         <v>98820079</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F75" s="2" t="s">
         <v>17</v>
@@ -4032,7 +4045,7 @@
     </row>
     <row r="76" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A76" s="3" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B76" s="12">
         <v>91732779</v>
@@ -4041,10 +4054,10 @@
         <v>98820079</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F76" s="2" t="s">
         <v>17</v>
@@ -4073,7 +4086,7 @@
     </row>
     <row r="77" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A77" s="3" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B77" s="12">
         <v>91732789</v>
@@ -4082,10 +4095,10 @@
         <v>98820079</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F77" s="2" t="s">
         <v>17</v>
@@ -4114,7 +4127,7 @@
     </row>
     <row r="78" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A78" s="3" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B78" s="12">
         <v>91546253</v>
@@ -4123,10 +4136,10 @@
         <v>98820079</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E78" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F78" s="2" t="s">
         <v>17</v>
@@ -4155,7 +4168,7 @@
     </row>
     <row r="79" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A79" s="3" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B79" s="13">
         <v>91732816</v>
@@ -4164,10 +4177,10 @@
         <v>98820079</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F79" s="2" t="s">
         <v>17</v>
@@ -4196,7 +4209,7 @@
     </row>
     <row r="80" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A80" s="3" t="s">
-        <v>93</v>
+        <v>74</v>
       </c>
       <c r="B80" s="13">
         <v>91546325</v>
@@ -4205,10 +4218,10 @@
         <v>98820079</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F80" s="2" t="s">
         <v>17</v>
@@ -4237,7 +4250,7 @@
     </row>
     <row r="81" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A81" s="3" t="s">
-        <v>94</v>
+        <v>75</v>
       </c>
       <c r="B81" s="13">
         <v>91732805</v>
@@ -4246,10 +4259,10 @@
         <v>98820079</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F81" s="2" t="s">
         <v>17</v>
@@ -4278,7 +4291,7 @@
     </row>
     <row r="82" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A82" s="3" t="s">
-        <v>95</v>
+        <v>76</v>
       </c>
       <c r="B82" s="13">
         <v>91732800</v>
@@ -4287,10 +4300,10 @@
         <v>98820079</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E82" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="F82" s="2" t="s">
         <v>17</v>
@@ -4321,17 +4334,17 @@
       <c r="A83" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B83" s="2">
+      <c r="B83" s="13">
         <v>98819619</v>
       </c>
       <c r="C83" s="2">
         <v>98820079</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>78</v>
+        <v>59</v>
       </c>
       <c r="F83" s="2" t="s">
         <v>15</v>
@@ -4339,7 +4352,7 @@
       <c r="G83" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H83" s="2" t="s">
+      <c r="H83" s="13" t="s">
         <v>13</v>
       </c>
       <c r="I83" s="4">
@@ -4349,28 +4362,30 @@
         <v>46162</v>
       </c>
       <c r="K83" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="L83" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="L83" s="2">
+        <v>1</v>
+      </c>
       <c r="M83" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="84" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A84" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B84" s="2">
+      <c r="B84" s="13">
         <v>98819621</v>
       </c>
       <c r="C84" s="2">
         <v>98820079</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>78</v>
+        <v>59</v>
       </c>
       <c r="F84" s="2" t="s">
         <v>12</v>
@@ -4378,7 +4393,7 @@
       <c r="G84" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H84" s="2" t="s">
+      <c r="H84" s="13" t="s">
         <v>13</v>
       </c>
       <c r="I84" s="4">
@@ -4388,28 +4403,30 @@
         <v>46162</v>
       </c>
       <c r="K84" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="L84" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="L84" s="2">
+        <v>2</v>
+      </c>
       <c r="M84" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="85" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A85" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B85" s="2">
+      <c r="B85" s="13">
         <v>98820081</v>
       </c>
       <c r="C85" s="3" t="s">
         <v>4</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>79</v>
+        <v>60</v>
       </c>
       <c r="F85" s="2" t="s">
         <v>35</v>
@@ -4417,7 +4434,7 @@
       <c r="G85" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H85" s="2" t="s">
+      <c r="H85" s="13" t="s">
         <v>7</v>
       </c>
       <c r="I85" s="4">
@@ -4438,17 +4455,17 @@
       <c r="A86" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B86" s="2">
+      <c r="B86" s="13">
         <v>98820079</v>
       </c>
       <c r="C86" s="3" t="s">
         <v>4</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>79</v>
+        <v>60</v>
       </c>
       <c r="F86" s="2" t="s">
         <v>35</v>
@@ -4456,7 +4473,7 @@
       <c r="G86" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H86" s="2" t="s">
+      <c r="H86" s="13" t="s">
         <v>8</v>
       </c>
       <c r="I86" s="4">
@@ -4477,17 +4494,17 @@
       <c r="A87" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B87" s="3" t="s">
+      <c r="B87" s="14" t="s">
         <v>4</v>
       </c>
       <c r="C87" s="3" t="s">
         <v>4</v>
       </c>
       <c r="D87" s="3" t="s">
-        <v>75</v>
+        <v>56</v>
       </c>
       <c r="E87" s="3" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="F87" s="2" t="s">
         <v>39</v>
@@ -4495,7 +4512,7 @@
       <c r="G87" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H87" s="2" t="s">
+      <c r="H87" s="13" t="s">
         <v>3</v>
       </c>
       <c r="I87" s="4">

</xml_diff>

<commit_message>
Last AMR devices installed
</commit_message>
<xml_diff>
--- a/EVG_Lake_Michelle_Meter_Hierarchy_2026-07-03.xlsx
+++ b/EVG_Lake_Michelle_Meter_Hierarchy_2026-07-03.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://voltano-my.sharepoint.com/personal/ruan_vh_voltano_com/Documents/Desktop/Voltano/Clients/Evergreen/Lake Michelle Noordhoek/Site Management/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="643" documentId="8_{E5281369-C957-4F01-BD7F-34BF193967CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2B5F2B9B-1969-4B1B-9C53-BFD42DB28BFE}"/>
+  <xr:revisionPtr revIDLastSave="693" documentId="8_{E5281369-C957-4F01-BD7F-34BF193967CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2B0664CC-0C8C-4DAC-9E29-A7FA8840D5D1}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{AE166FFD-83CC-4E71-A293-C6082B1A6C83}"/>
+    <workbookView xWindow="71880" yWindow="-1530" windowWidth="29040" windowHeight="15720" xr2:uid="{AE166FFD-83CC-4E71-A293-C6082B1A6C83}"/>
   </bookViews>
   <sheets>
     <sheet name="Elec" sheetId="1" r:id="rId1"/>
@@ -182,30 +182,6 @@
     <t>050</t>
   </si>
   <si>
-    <t>073</t>
-  </si>
-  <si>
-    <t>074</t>
-  </si>
-  <si>
-    <t>075</t>
-  </si>
-  <si>
-    <t>076</t>
-  </si>
-  <si>
-    <t>077</t>
-  </si>
-  <si>
-    <t>078</t>
-  </si>
-  <si>
-    <t>079</t>
-  </si>
-  <si>
-    <t>080</t>
-  </si>
-  <si>
     <t>Manufacturer</t>
   </si>
   <si>
@@ -447,6 +423,30 @@
   </si>
   <si>
     <t>11</t>
+  </si>
+  <si>
+    <t>006</t>
+  </si>
+  <si>
+    <t>005</t>
+  </si>
+  <si>
+    <t>007</t>
+  </si>
+  <si>
+    <t>008</t>
+  </si>
+  <si>
+    <t>001</t>
+  </si>
+  <si>
+    <t>002</t>
+  </si>
+  <si>
+    <t>003</t>
+  </si>
+  <si>
+    <t>004</t>
   </si>
 </sst>
 </file>
@@ -992,13 +992,13 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>5</v>
@@ -1007,27 +1007,27 @@
         <v>2</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="K1" s="10" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="L1" s="10" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="M1" s="10" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A2" s="3" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="B2" s="13">
         <v>91732777</v>
@@ -1036,10 +1036,10 @@
         <v>98820079</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>17</v>
@@ -1068,7 +1068,7 @@
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="B3" s="13">
         <v>91732837</v>
@@ -1077,10 +1077,10 @@
         <v>98820079</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>17</v>
@@ -1109,7 +1109,7 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="B4" s="13">
         <v>91733081</v>
@@ -1118,10 +1118,10 @@
         <v>98820079</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>17</v>
@@ -1150,7 +1150,7 @@
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A5" s="3" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="B5" s="13">
         <v>91732799</v>
@@ -1159,10 +1159,10 @@
         <v>98820079</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>17</v>
@@ -1191,7 +1191,7 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A6" s="3" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="B6" s="13">
         <v>91546302</v>
@@ -1200,10 +1200,10 @@
         <v>98820079</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>17</v>
@@ -1232,7 +1232,7 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A7" s="3" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="B7" s="13">
         <v>91732803</v>
@@ -1241,10 +1241,10 @@
         <v>98820079</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>17</v>
@@ -1273,7 +1273,7 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A8" s="3" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="B8" s="13">
         <v>91546328</v>
@@ -1282,10 +1282,10 @@
         <v>98820079</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>17</v>
@@ -1314,7 +1314,7 @@
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A9" s="3" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="B9" s="13">
         <v>91546327</v>
@@ -1323,10 +1323,10 @@
         <v>98820079</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>17</v>
@@ -1355,7 +1355,7 @@
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A10" s="3" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="B10" s="13">
         <v>91546252</v>
@@ -1364,10 +1364,10 @@
         <v>98820079</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>17</v>
@@ -1396,7 +1396,7 @@
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A11" s="3" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="B11" s="13">
         <v>91732812</v>
@@ -1405,10 +1405,10 @@
         <v>98820079</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>17</v>
@@ -1437,7 +1437,7 @@
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A12" s="3" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="B12" s="13">
         <v>91546326</v>
@@ -1446,10 +1446,10 @@
         <v>98820079</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>17</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A13" s="3" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="B13" s="13">
         <v>91732785</v>
@@ -1487,10 +1487,10 @@
         <v>98820079</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>17</v>
@@ -1519,7 +1519,7 @@
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A14" s="3" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="B14" s="13">
         <v>91732797</v>
@@ -1528,10 +1528,10 @@
         <v>98820081</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>17</v>
@@ -1560,7 +1560,7 @@
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A15" s="3" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="B15" s="13">
         <v>91732835</v>
@@ -1569,10 +1569,10 @@
         <v>98820081</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>17</v>
@@ -1601,7 +1601,7 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A16" s="3" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="B16" s="13">
         <v>91546283</v>
@@ -1610,10 +1610,10 @@
         <v>98820081</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>17</v>
@@ -1642,7 +1642,7 @@
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A17" s="3" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="B17" s="13">
         <v>91732806</v>
@@ -1651,10 +1651,10 @@
         <v>98820081</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>17</v>
@@ -1683,7 +1683,7 @@
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A18" s="3" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="B18" s="13">
         <v>91732775</v>
@@ -1692,10 +1692,10 @@
         <v>98820081</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>17</v>
@@ -1724,19 +1724,19 @@
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A19" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="B19" s="2">
+        <v>134</v>
+      </c>
+      <c r="B19" s="13">
         <v>91732809</v>
       </c>
       <c r="C19" s="2">
         <v>98820079</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>17</v>
@@ -1744,7 +1744,7 @@
       <c r="G19" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H19" s="2" t="s">
+      <c r="H19" s="13" t="s">
         <v>34</v>
       </c>
       <c r="I19" s="4">
@@ -1754,28 +1754,30 @@
         <v>46162</v>
       </c>
       <c r="K19" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="L19" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="L19" s="2">
+        <v>4</v>
+      </c>
       <c r="M19" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A20" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="B20" s="2">
+        <v>133</v>
+      </c>
+      <c r="B20" s="13">
         <v>91732788</v>
       </c>
       <c r="C20" s="2">
         <v>98820079</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>17</v>
@@ -1783,7 +1785,7 @@
       <c r="G20" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="H20" s="2" t="s">
+      <c r="H20" s="13" t="s">
         <v>34</v>
       </c>
       <c r="I20" s="4">
@@ -1793,28 +1795,30 @@
         <v>46162</v>
       </c>
       <c r="K20" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="L20" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="L20" s="2">
+        <v>3</v>
+      </c>
       <c r="M20" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A21" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="B21" s="2">
+        <v>132</v>
+      </c>
+      <c r="B21" s="13">
         <v>91546333</v>
       </c>
       <c r="C21" s="2">
         <v>98820079</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>17</v>
@@ -1822,7 +1826,7 @@
       <c r="G21" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="H21" s="2" t="s">
+      <c r="H21" s="13" t="s">
         <v>34</v>
       </c>
       <c r="I21" s="4">
@@ -1832,28 +1836,30 @@
         <v>46162</v>
       </c>
       <c r="K21" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="L21" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="L21" s="2">
+        <v>2</v>
+      </c>
       <c r="M21" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A22" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="B22" s="2">
+        <v>131</v>
+      </c>
+      <c r="B22" s="13">
         <v>91732814</v>
       </c>
       <c r="C22" s="2">
         <v>98820079</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>17</v>
@@ -1861,7 +1867,7 @@
       <c r="G22" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H22" s="2" t="s">
+      <c r="H22" s="13" t="s">
         <v>34</v>
       </c>
       <c r="I22" s="4">
@@ -1871,16 +1877,18 @@
         <v>46162</v>
       </c>
       <c r="K22" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="L22" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="L22" s="2">
+        <v>1</v>
+      </c>
       <c r="M22" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A23" s="3" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="B23" s="13">
         <v>91732831</v>
@@ -1889,10 +1897,10 @@
         <v>98820081</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F23" s="2" t="s">
         <v>17</v>
@@ -1921,7 +1929,7 @@
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A24" s="3" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="B24" s="13">
         <v>91732781</v>
@@ -1930,10 +1938,10 @@
         <v>98820081</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>17</v>
@@ -1962,7 +1970,7 @@
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A25" s="3" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="B25" s="13">
         <v>91732815</v>
@@ -1971,10 +1979,10 @@
         <v>98820081</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>17</v>
@@ -2003,7 +2011,7 @@
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A26" s="3" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="B26" s="13">
         <v>91732780</v>
@@ -2012,10 +2020,10 @@
         <v>98820081</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F26" s="2" t="s">
         <v>17</v>
@@ -2044,7 +2052,7 @@
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A27" s="3" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="B27" s="13">
         <v>91732841</v>
@@ -2053,10 +2061,10 @@
         <v>98820081</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F27" s="2" t="s">
         <v>17</v>
@@ -2085,19 +2093,19 @@
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A28" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B28" s="4">
+        <v>130</v>
+      </c>
+      <c r="B28" s="12">
         <v>91732795</v>
       </c>
       <c r="C28" s="2">
         <v>98820079</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F28" s="2" t="s">
         <v>17</v>
@@ -2105,7 +2113,7 @@
       <c r="G28" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="H28" s="2" t="s">
+      <c r="H28" s="13" t="s">
         <v>33</v>
       </c>
       <c r="I28" s="4">
@@ -2115,28 +2123,30 @@
         <v>46162</v>
       </c>
       <c r="K28" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="L28" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="L28" s="2">
+        <v>4</v>
+      </c>
       <c r="M28" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A29" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="B29" s="4">
+        <v>129</v>
+      </c>
+      <c r="B29" s="12">
         <v>91546331</v>
       </c>
       <c r="C29" s="2">
         <v>98820079</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F29" s="2" t="s">
         <v>17</v>
@@ -2144,7 +2154,7 @@
       <c r="G29" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="H29" s="2" t="s">
+      <c r="H29" s="13" t="s">
         <v>33</v>
       </c>
       <c r="I29" s="4">
@@ -2154,28 +2164,30 @@
         <v>46162</v>
       </c>
       <c r="K29" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="L29" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="L29" s="2">
+        <v>3</v>
+      </c>
       <c r="M29" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A30" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="B30" s="4">
+        <v>127</v>
+      </c>
+      <c r="B30" s="12">
         <v>91732836</v>
       </c>
       <c r="C30" s="2">
         <v>98820079</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F30" s="2" t="s">
         <v>17</v>
@@ -2183,7 +2195,7 @@
       <c r="G30" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="H30" s="2" t="s">
+      <c r="H30" s="13" t="s">
         <v>33</v>
       </c>
       <c r="I30" s="4">
@@ -2193,28 +2205,30 @@
         <v>46162</v>
       </c>
       <c r="K30" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="L30" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="L30" s="2">
+        <v>2</v>
+      </c>
       <c r="M30" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A31" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="B31" s="4">
+        <v>128</v>
+      </c>
+      <c r="B31" s="12">
         <v>91732802</v>
       </c>
       <c r="C31" s="2">
         <v>98820079</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F31" s="2" t="s">
         <v>17</v>
@@ -2222,7 +2236,7 @@
       <c r="G31" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="H31" s="2" t="s">
+      <c r="H31" s="13" t="s">
         <v>33</v>
       </c>
       <c r="I31" s="4">
@@ -2232,11 +2246,13 @@
         <v>46162</v>
       </c>
       <c r="K31" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="L31" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="L31" s="2">
+        <v>1</v>
+      </c>
       <c r="M31" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.45">
@@ -2250,10 +2266,10 @@
         <v>98820081</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="F32" s="2" t="s">
         <v>12</v>
@@ -2282,7 +2298,7 @@
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A33" s="3" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="B33" s="13">
         <v>91546282</v>
@@ -2291,10 +2307,10 @@
         <v>98820079</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F33" s="2" t="s">
         <v>17</v>
@@ -2323,7 +2339,7 @@
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A34" s="3" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="B34" s="13">
         <v>91732791</v>
@@ -2332,10 +2348,10 @@
         <v>98820079</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F34" s="2" t="s">
         <v>17</v>
@@ -2364,7 +2380,7 @@
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A35" s="3" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="B35" s="13">
         <v>91732818</v>
@@ -2373,10 +2389,10 @@
         <v>98820079</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F35" s="2" t="s">
         <v>17</v>
@@ -2405,7 +2421,7 @@
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A36" s="3" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="B36" s="13">
         <v>91732782</v>
@@ -2414,10 +2430,10 @@
         <v>98820079</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F36" s="2" t="s">
         <v>17</v>
@@ -2446,7 +2462,7 @@
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A37" s="3" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="B37" s="13">
         <v>91546307</v>
@@ -2455,10 +2471,10 @@
         <v>98820079</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F37" s="2" t="s">
         <v>17</v>
@@ -2487,7 +2503,7 @@
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A38" s="3" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="B38" s="13">
         <v>91732842</v>
@@ -2496,10 +2512,10 @@
         <v>98820081</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F38" s="2" t="s">
         <v>17</v>
@@ -2528,7 +2544,7 @@
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A39" s="3" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="B39" s="13">
         <v>91732793</v>
@@ -2537,10 +2553,10 @@
         <v>98820081</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F39" s="2" t="s">
         <v>17</v>
@@ -2569,7 +2585,7 @@
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A40" s="3" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="B40" s="13">
         <v>91732840</v>
@@ -2578,10 +2594,10 @@
         <v>98820081</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F40" s="2" t="s">
         <v>17</v>
@@ -2610,7 +2626,7 @@
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A41" s="3" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="B41" s="13">
         <v>91732817</v>
@@ -2619,10 +2635,10 @@
         <v>98820081</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F41" s="2" t="s">
         <v>17</v>
@@ -2651,7 +2667,7 @@
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A42" s="3" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="B42" s="13">
         <v>91732792</v>
@@ -2660,10 +2676,10 @@
         <v>98820081</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F42" s="2" t="s">
         <v>17</v>
@@ -2692,7 +2708,7 @@
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A43" s="3" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="B43" s="13">
         <v>91732796</v>
@@ -2701,10 +2717,10 @@
         <v>98820081</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F43" s="2" t="s">
         <v>17</v>
@@ -2733,7 +2749,7 @@
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A44" s="3" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="B44" s="13">
         <v>91546227</v>
@@ -2742,10 +2758,10 @@
         <v>98820079</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F44" s="2" t="s">
         <v>17</v>
@@ -2774,7 +2790,7 @@
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A45" s="3" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="B45" s="13">
         <v>91732786</v>
@@ -2783,10 +2799,10 @@
         <v>98820079</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F45" s="2" t="s">
         <v>17</v>
@@ -2815,7 +2831,7 @@
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A46" s="3" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="B46" s="13">
         <v>91732808</v>
@@ -2824,10 +2840,10 @@
         <v>98820079</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F46" s="2" t="s">
         <v>17</v>
@@ -2856,7 +2872,7 @@
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A47" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B47" s="13">
         <v>91546277</v>
@@ -2865,10 +2881,10 @@
         <v>98820079</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F47" s="2" t="s">
         <v>17</v>
@@ -2897,7 +2913,7 @@
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A48" s="3" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="B48" s="13">
         <v>91732798</v>
@@ -2906,10 +2922,10 @@
         <v>98820079</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F48" s="2" t="s">
         <v>17</v>
@@ -2938,7 +2954,7 @@
     </row>
     <row r="49" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A49" s="3" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="B49" s="13">
         <v>91732794</v>
@@ -2947,10 +2963,10 @@
         <v>98820081</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F49" s="2" t="s">
         <v>17</v>
@@ -2979,7 +2995,7 @@
     </row>
     <row r="50" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A50" s="3" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="B50" s="13">
         <v>91732774</v>
@@ -2988,10 +3004,10 @@
         <v>98820081</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F50" s="2" t="s">
         <v>17</v>
@@ -3020,7 +3036,7 @@
     </row>
     <row r="51" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A51" s="3" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="B51" s="13">
         <v>91732776</v>
@@ -3029,10 +3045,10 @@
         <v>98820081</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F51" s="2" t="s">
         <v>17</v>
@@ -3061,7 +3077,7 @@
     </row>
     <row r="52" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A52" s="3" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="B52" s="13">
         <v>91732801</v>
@@ -3070,10 +3086,10 @@
         <v>98820081</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F52" s="2" t="s">
         <v>17</v>
@@ -3102,7 +3118,7 @@
     </row>
     <row r="53" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A53" s="3" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="B53" s="13">
         <v>91732784</v>
@@ -3111,10 +3127,10 @@
         <v>98820081</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F53" s="2" t="s">
         <v>17</v>
@@ -3143,7 +3159,7 @@
     </row>
     <row r="54" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A54" s="3" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="B54" s="13">
         <v>91732790</v>
@@ -3152,10 +3168,10 @@
         <v>98820081</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F54" s="2" t="s">
         <v>17</v>
@@ -3184,7 +3200,7 @@
     </row>
     <row r="55" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A55" s="3" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="B55" s="13">
         <v>91546303</v>
@@ -3193,10 +3209,10 @@
         <v>98820079</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F55" s="2" t="s">
         <v>17</v>
@@ -3225,7 +3241,7 @@
     </row>
     <row r="56" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A56" s="3" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="B56" s="13">
         <v>91546278</v>
@@ -3234,10 +3250,10 @@
         <v>98820079</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F56" s="2" t="s">
         <v>17</v>
@@ -3266,7 +3282,7 @@
     </row>
     <row r="57" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A57" s="3" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="B57" s="13">
         <v>91542774</v>
@@ -3275,10 +3291,10 @@
         <v>98820079</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F57" s="2" t="s">
         <v>17</v>
@@ -3307,7 +3323,7 @@
     </row>
     <row r="58" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A58" s="3" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="B58" s="13">
         <v>91732833</v>
@@ -3316,10 +3332,10 @@
         <v>98820079</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F58" s="2" t="s">
         <v>17</v>
@@ -3348,7 +3364,7 @@
     </row>
     <row r="59" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A59" s="3" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="B59" s="13">
         <v>91732778</v>
@@ -3357,10 +3373,10 @@
         <v>98820079</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F59" s="2" t="s">
         <v>17</v>
@@ -3389,7 +3405,7 @@
     </row>
     <row r="60" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A60" s="3" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="B60" s="13">
         <v>91546300</v>
@@ -3398,10 +3414,10 @@
         <v>98820081</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F60" s="2" t="s">
         <v>17</v>
@@ -3430,7 +3446,7 @@
     </row>
     <row r="61" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A61" s="3" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="B61" s="13">
         <v>91732839</v>
@@ -3439,10 +3455,10 @@
         <v>98820081</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F61" s="2" t="s">
         <v>17</v>
@@ -3471,7 +3487,7 @@
     </row>
     <row r="62" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A62" s="3" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="B62" s="13">
         <v>91546308</v>
@@ -3480,10 +3496,10 @@
         <v>98820081</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F62" s="2" t="s">
         <v>17</v>
@@ -3512,7 +3528,7 @@
     </row>
     <row r="63" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A63" s="3" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="B63" s="13">
         <v>91732813</v>
@@ -3521,10 +3537,10 @@
         <v>98820081</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F63" s="2" t="s">
         <v>17</v>
@@ -3553,7 +3569,7 @@
     </row>
     <row r="64" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A64" s="3" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="B64" s="13">
         <v>91732804</v>
@@ -3562,10 +3578,10 @@
         <v>98820079</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F64" s="2" t="s">
         <v>17</v>
@@ -3594,7 +3610,7 @@
     </row>
     <row r="65" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A65" s="3" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="B65" s="13">
         <v>91546301</v>
@@ -3603,10 +3619,10 @@
         <v>98820079</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F65" s="2" t="s">
         <v>17</v>
@@ -3635,7 +3651,7 @@
     </row>
     <row r="66" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A66" s="3" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="B66" s="13">
         <v>91732807</v>
@@ -3644,10 +3660,10 @@
         <v>98820079</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F66" s="2" t="s">
         <v>17</v>
@@ -3676,7 +3692,7 @@
     </row>
     <row r="67" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A67" s="3" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="B67" s="13">
         <v>91546332</v>
@@ -3685,10 +3701,10 @@
         <v>98820079</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F67" s="2" t="s">
         <v>17</v>
@@ -3717,7 +3733,7 @@
     </row>
     <row r="68" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A68" s="3" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="B68" s="13">
         <v>91546306</v>
@@ -3726,10 +3742,10 @@
         <v>98820079</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F68" s="2" t="s">
         <v>17</v>
@@ -3758,7 +3774,7 @@
     </row>
     <row r="69" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A69" s="3" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="B69" s="13">
         <v>91732811</v>
@@ -3767,10 +3783,10 @@
         <v>98820079</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F69" s="2" t="s">
         <v>17</v>
@@ -3799,7 +3815,7 @@
     </row>
     <row r="70" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A70" s="3" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="B70" s="13">
         <v>91732773</v>
@@ -3808,10 +3824,10 @@
         <v>98820081</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F70" s="2" t="s">
         <v>17</v>
@@ -3840,7 +3856,7 @@
     </row>
     <row r="71" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A71" s="3" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="B71" s="13">
         <v>91732810</v>
@@ -3849,10 +3865,10 @@
         <v>98820081</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F71" s="2" t="s">
         <v>17</v>
@@ -3881,7 +3897,7 @@
     </row>
     <row r="72" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A72" s="3" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="B72" s="13">
         <v>91732787</v>
@@ -3890,10 +3906,10 @@
         <v>98820081</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F72" s="2" t="s">
         <v>17</v>
@@ -3922,7 +3938,7 @@
     </row>
     <row r="73" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A73" s="3" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="B73" s="13">
         <v>91732771</v>
@@ -3931,10 +3947,10 @@
         <v>98820081</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F73" s="2" t="s">
         <v>17</v>
@@ -3972,10 +3988,10 @@
         <v>98820079</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F74" s="2" t="s">
         <v>17</v>
@@ -4013,10 +4029,10 @@
         <v>98820079</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F75" s="2" t="s">
         <v>17</v>
@@ -4054,10 +4070,10 @@
         <v>98820079</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F76" s="2" t="s">
         <v>17</v>
@@ -4095,10 +4111,10 @@
         <v>98820079</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F77" s="2" t="s">
         <v>17</v>
@@ -4136,10 +4152,10 @@
         <v>98820079</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E78" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F78" s="2" t="s">
         <v>17</v>
@@ -4177,10 +4193,10 @@
         <v>98820079</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F79" s="2" t="s">
         <v>17</v>
@@ -4209,7 +4225,7 @@
     </row>
     <row r="80" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A80" s="3" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="B80" s="13">
         <v>91546325</v>
@@ -4218,10 +4234,10 @@
         <v>98820079</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F80" s="2" t="s">
         <v>17</v>
@@ -4250,7 +4266,7 @@
     </row>
     <row r="81" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A81" s="3" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="B81" s="13">
         <v>91732805</v>
@@ -4259,10 +4275,10 @@
         <v>98820079</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F81" s="2" t="s">
         <v>17</v>
@@ -4291,7 +4307,7 @@
     </row>
     <row r="82" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A82" s="3" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="B82" s="13">
         <v>91732800</v>
@@ -4300,10 +4316,10 @@
         <v>98820079</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E82" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F82" s="2" t="s">
         <v>17</v>
@@ -4341,10 +4357,10 @@
         <v>98820079</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="F83" s="2" t="s">
         <v>15</v>
@@ -4382,10 +4398,10 @@
         <v>98820079</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="F84" s="2" t="s">
         <v>12</v>
@@ -4423,10 +4439,10 @@
         <v>4</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="F85" s="2" t="s">
         <v>35</v>
@@ -4446,7 +4462,9 @@
       <c r="K85" s="11" t="b">
         <v>1</v>
       </c>
-      <c r="L85" s="2"/>
+      <c r="L85" s="2">
+        <v>1</v>
+      </c>
       <c r="M85" s="11" t="b">
         <v>1</v>
       </c>
@@ -4462,10 +4480,10 @@
         <v>4</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="F86" s="2" t="s">
         <v>35</v>
@@ -4485,7 +4503,9 @@
       <c r="K86" s="11" t="b">
         <v>1</v>
       </c>
-      <c r="L86" s="2"/>
+      <c r="L86" s="2">
+        <v>1</v>
+      </c>
       <c r="M86" s="11" t="b">
         <v>1</v>
       </c>
@@ -4501,10 +4521,10 @@
         <v>4</v>
       </c>
       <c r="D87" s="3" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="E87" s="3" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="F87" s="2" t="s">
         <v>39</v>

</xml_diff>